<commit_message>
[47]  C009: Valorizzata la colonna J [48]  C009: Valorizzata la colonna J [191] C011: Valorizzata la colonna K [376] C011: Valorizzata la colonna K [425] C009: Valorizzata la colonna J
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#GASNETGROUPXX/gasnet/SaniPocket/V1.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#GASNETGROUPXX/gasnet/SaniPocket/V1.0/report-checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\simone.bettini\Desktop\temp\20260310_labelling_nazionale_LAB_LDO_RAD_RAP_RSA\SUBMISSION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFAE670D-9F1E-4C75-B1CB-622DC14F44F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E245846C-7BDE-4EEB-9A39-C8A7016C6CCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-135" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -2820,6 +2820,10 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -2838,10 +2842,6 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal 2" xfId="1" xr:uid="{565105C8-FFD6-432C-8B2E-BD1D172FCD26}"/>
@@ -4279,6 +4279,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:W745"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
@@ -4327,10 +4328,10 @@
         <v>12</v>
       </c>
       <c r="B2" s="53"/>
-      <c r="C2" s="60" t="s">
+      <c r="C2" s="54" t="s">
         <v>617</v>
       </c>
-      <c r="D2" s="61"/>
+      <c r="D2" s="55"/>
       <c r="F2" s="26"/>
       <c r="G2" s="26"/>
       <c r="H2" s="26"/>
@@ -4351,14 +4352,14 @@
       <c r="W2" s="30"/>
     </row>
     <row r="3" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="54" t="s">
+      <c r="A3" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="55"/>
-      <c r="C3" s="60" t="s">
+      <c r="B3" s="57"/>
+      <c r="C3" s="54" t="s">
         <v>614</v>
       </c>
-      <c r="D3" s="61"/>
+      <c r="D3" s="55"/>
       <c r="F3" s="26"/>
       <c r="G3" s="26"/>
       <c r="H3" s="26"/>
@@ -4379,12 +4380,12 @@
       <c r="W3" s="30"/>
     </row>
     <row r="4" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="56"/>
-      <c r="B4" s="57"/>
-      <c r="C4" s="60" t="s">
+      <c r="A4" s="58"/>
+      <c r="B4" s="59"/>
+      <c r="C4" s="54" t="s">
         <v>615</v>
       </c>
-      <c r="D4" s="61"/>
+      <c r="D4" s="55"/>
       <c r="F4" s="26"/>
       <c r="G4" s="26"/>
       <c r="H4" s="26"/>
@@ -4405,12 +4406,12 @@
       <c r="W4" s="30"/>
     </row>
     <row r="5" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="58"/>
-      <c r="B5" s="59"/>
-      <c r="C5" s="60" t="s">
+      <c r="A5" s="60"/>
+      <c r="B5" s="61"/>
+      <c r="C5" s="54" t="s">
         <v>616</v>
       </c>
-      <c r="D5" s="61"/>
+      <c r="D5" s="55"/>
       <c r="F5" s="26"/>
       <c r="G5" s="26"/>
       <c r="H5" s="26"/>
@@ -4567,7 +4568,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="36">
         <v>4</v>
       </c>
@@ -4627,7 +4628,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="24">
         <v>28</v>
       </c>
@@ -4696,7 +4697,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="24">
         <v>29</v>
       </c>
@@ -4765,7 +4766,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="24">
         <v>30</v>
       </c>
@@ -4830,7 +4831,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="24">
         <v>31</v>
       </c>
@@ -4899,7 +4900,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" ht="13.5" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="24">
         <v>32</v>
       </c>
@@ -4968,7 +4969,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="24">
         <v>33</v>
       </c>
@@ -5033,7 +5034,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="24">
         <v>34</v>
       </c>
@@ -5098,7 +5099,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="24">
         <v>35</v>
       </c>
@@ -5163,7 +5164,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="19" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="24">
         <v>36</v>
       </c>
@@ -5232,7 +5233,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="20" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="24">
         <v>37</v>
       </c>
@@ -5301,7 +5302,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="24">
         <v>38</v>
       </c>
@@ -5366,7 +5367,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="22" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="24">
         <v>39</v>
       </c>
@@ -5435,7 +5436,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="24">
         <v>40</v>
       </c>
@@ -5504,7 +5505,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="24" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="24">
         <v>41</v>
       </c>
@@ -5569,7 +5570,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="24">
         <v>42</v>
       </c>
@@ -5634,7 +5635,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="26" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="24">
         <v>43</v>
       </c>
@@ -5699,7 +5700,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="27" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="24">
         <v>44</v>
       </c>
@@ -5764,7 +5765,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="28" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="24">
         <v>45</v>
       </c>
@@ -5829,7 +5830,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="24">
         <v>46</v>
       </c>
@@ -5919,7 +5920,7 @@
         <v>440</v>
       </c>
       <c r="J30" s="41" t="s">
-        <v>440</v>
+        <v>62</v>
       </c>
       <c r="K30" s="41" t="s">
         <v>440</v>
@@ -5984,7 +5985,7 @@
         <v>440</v>
       </c>
       <c r="J31" s="41" t="s">
-        <v>440</v>
+        <v>62</v>
       </c>
       <c r="K31" s="41" t="s">
         <v>440</v>
@@ -6024,7 +6025,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="32" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="24">
         <v>49</v>
       </c>
@@ -6089,7 +6090,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="33" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A33" s="24">
         <v>50</v>
       </c>
@@ -6154,7 +6155,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="34" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34" s="24">
         <v>51</v>
       </c>
@@ -6219,7 +6220,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="35" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A35" s="24">
         <v>53</v>
       </c>
@@ -6288,7 +6289,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="36" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="24">
         <v>55</v>
       </c>
@@ -6357,7 +6358,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="37" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="24">
         <v>56</v>
       </c>
@@ -6426,7 +6427,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="38" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38" s="24">
         <v>57</v>
       </c>
@@ -6495,7 +6496,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A39" s="24">
         <v>59</v>
       </c>
@@ -6564,7 +6565,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="40" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A40" s="24">
         <v>60</v>
       </c>
@@ -6633,7 +6634,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="41" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A41" s="24">
         <v>61</v>
       </c>
@@ -6702,7 +6703,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="42" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A42" s="24">
         <v>62</v>
       </c>
@@ -6771,7 +6772,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="43" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A43" s="24">
         <v>64</v>
       </c>
@@ -6840,7 +6841,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="44" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A44" s="24">
         <v>66</v>
       </c>
@@ -6909,7 +6910,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A45" s="24">
         <v>67</v>
       </c>
@@ -6978,7 +6979,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A46" s="24">
         <v>68</v>
       </c>
@@ -7047,7 +7048,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="47" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="24">
         <v>69</v>
       </c>
@@ -7116,7 +7117,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="48" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A48" s="24">
         <v>70</v>
       </c>
@@ -7185,7 +7186,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="49" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A49" s="24">
         <v>71</v>
       </c>
@@ -7254,7 +7255,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="50" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A50" s="24">
         <v>72</v>
       </c>
@@ -7323,7 +7324,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="51" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A51" s="24">
         <v>73</v>
       </c>
@@ -7392,7 +7393,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="52" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A52" s="24">
         <v>74</v>
       </c>
@@ -7461,7 +7462,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="53" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A53" s="24">
         <v>76</v>
       </c>
@@ -7530,7 +7531,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="54" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="24">
         <v>78</v>
       </c>
@@ -7599,7 +7600,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="55" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A55" s="24">
         <v>79</v>
       </c>
@@ -7668,7 +7669,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="56" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A56" s="24">
         <v>80</v>
       </c>
@@ -7737,7 +7738,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="57" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A57" s="24">
         <v>81</v>
       </c>
@@ -7806,7 +7807,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="58" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A58" s="24">
         <v>83</v>
       </c>
@@ -7875,7 +7876,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="59" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A59" s="24">
         <v>84</v>
       </c>
@@ -7944,7 +7945,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="60" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A60" s="24">
         <v>85</v>
       </c>
@@ -8013,7 +8014,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="61" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A61" s="24">
         <v>86</v>
       </c>
@@ -8082,7 +8083,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="62" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A62" s="24">
         <v>87</v>
       </c>
@@ -8151,7 +8152,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="63" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A63" s="24">
         <v>88</v>
       </c>
@@ -8220,7 +8221,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="64" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A64" s="24">
         <v>89</v>
       </c>
@@ -8289,7 +8290,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="65" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A65" s="24">
         <v>90</v>
       </c>
@@ -8358,7 +8359,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="66" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A66" s="24">
         <v>91</v>
       </c>
@@ -8427,7 +8428,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="67" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A67" s="24">
         <v>92</v>
       </c>
@@ -8496,7 +8497,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="68" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A68" s="24">
         <v>93</v>
       </c>
@@ -8565,7 +8566,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="69" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A69" s="24">
         <v>95</v>
       </c>
@@ -8630,7 +8631,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="70" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A70" s="24">
         <v>97</v>
       </c>
@@ -8695,7 +8696,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="71" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A71" s="24">
         <v>98</v>
       </c>
@@ -8760,7 +8761,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="72" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A72" s="24">
         <v>99</v>
       </c>
@@ -8825,7 +8826,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="73" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A73" s="24">
         <v>100</v>
       </c>
@@ -8890,7 +8891,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="74" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A74" s="24">
         <v>101</v>
       </c>
@@ -8955,7 +8956,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="75" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A75" s="24">
         <v>102</v>
       </c>
@@ -9020,7 +9021,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="76" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A76" s="24">
         <v>103</v>
       </c>
@@ -9085,7 +9086,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="77" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A77" s="24">
         <v>104</v>
       </c>
@@ -9150,7 +9151,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="78" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A78" s="24">
         <v>105</v>
       </c>
@@ -9215,7 +9216,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="79" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A79" s="24">
         <v>106</v>
       </c>
@@ -9280,7 +9281,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="80" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A80" s="24">
         <v>108</v>
       </c>
@@ -9345,7 +9346,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="81" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A81" s="24">
         <v>110</v>
       </c>
@@ -9410,7 +9411,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="82" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A82" s="24">
         <v>111</v>
       </c>
@@ -9475,7 +9476,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="83" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A83" s="24">
         <v>112</v>
       </c>
@@ -9540,7 +9541,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="84" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A84" s="24">
         <v>113</v>
       </c>
@@ -9605,7 +9606,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="85" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A85" s="24">
         <v>114</v>
       </c>
@@ -9670,7 +9671,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="86" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A86" s="24">
         <v>115</v>
       </c>
@@ -9735,7 +9736,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="87" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A87" s="24">
         <v>116</v>
       </c>
@@ -9800,7 +9801,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="88" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A88" s="24">
         <v>117</v>
       </c>
@@ -9865,7 +9866,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="89" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A89" s="24">
         <v>118</v>
       </c>
@@ -9930,7 +9931,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="90" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A90" s="24">
         <v>119</v>
       </c>
@@ -9995,7 +9996,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="91" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A91" s="24">
         <v>120</v>
       </c>
@@ -10060,7 +10061,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="92" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A92" s="24">
         <v>121</v>
       </c>
@@ -10125,7 +10126,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="93" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A93" s="24">
         <v>123</v>
       </c>
@@ -10190,7 +10191,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="94" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A94" s="24">
         <v>125</v>
       </c>
@@ -10255,7 +10256,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="95" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A95" s="24">
         <v>126</v>
       </c>
@@ -10320,7 +10321,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="96" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A96" s="24">
         <v>127</v>
       </c>
@@ -10385,7 +10386,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="97" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A97" s="24">
         <v>128</v>
       </c>
@@ -10450,7 +10451,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="98" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A98" s="24">
         <v>129</v>
       </c>
@@ -10515,7 +10516,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="99" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A99" s="24">
         <v>130</v>
       </c>
@@ -10580,7 +10581,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="100" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A100" s="24">
         <v>131</v>
       </c>
@@ -10645,7 +10646,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="101" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A101" s="24">
         <v>132</v>
       </c>
@@ -10710,7 +10711,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="102" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A102" s="24">
         <v>133</v>
       </c>
@@ -10775,7 +10776,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="103" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A103" s="24">
         <v>134</v>
       </c>
@@ -10840,7 +10841,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="104" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A104" s="24">
         <v>135</v>
       </c>
@@ -10905,7 +10906,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="105" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A105" s="24">
         <v>136</v>
       </c>
@@ -10970,7 +10971,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="106" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A106" s="24">
         <v>137</v>
       </c>
@@ -11035,7 +11036,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="107" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A107" s="24">
         <v>138</v>
       </c>
@@ -11100,7 +11101,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="108" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A108" s="24">
         <v>139</v>
       </c>
@@ -11165,7 +11166,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="109" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A109" s="24">
         <v>140</v>
       </c>
@@ -11230,7 +11231,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="110" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A110" s="24">
         <v>141</v>
       </c>
@@ -11295,7 +11296,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="111" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A111" s="24">
         <v>142</v>
       </c>
@@ -11360,7 +11361,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="112" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A112" s="24">
         <v>143</v>
       </c>
@@ -11425,7 +11426,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="113" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A113" s="24">
         <v>144</v>
       </c>
@@ -11490,7 +11491,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="114" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A114" s="24">
         <v>145</v>
       </c>
@@ -11555,7 +11556,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="115" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A115" s="24">
         <v>146</v>
       </c>
@@ -11620,7 +11621,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="116" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A116" s="24">
         <v>152</v>
       </c>
@@ -11689,7 +11690,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="117" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A117" s="24">
         <v>154</v>
       </c>
@@ -11758,7 +11759,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="118" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A118" s="24">
         <v>155</v>
       </c>
@@ -11827,7 +11828,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="119" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A119" s="24">
         <v>156</v>
       </c>
@@ -11896,7 +11897,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="120" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A120" s="24">
         <v>159</v>
       </c>
@@ -11965,7 +11966,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="121" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A121" s="24">
         <v>160</v>
       </c>
@@ -12034,7 +12035,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="122" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A122" s="24">
         <v>161</v>
       </c>
@@ -12103,7 +12104,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="123" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A123" s="24">
         <v>162</v>
       </c>
@@ -12172,7 +12173,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="124" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A124" s="24">
         <v>163</v>
       </c>
@@ -12241,7 +12242,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="125" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A125" s="24">
         <v>164</v>
       </c>
@@ -12310,7 +12311,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="126" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A126" s="24">
         <v>165</v>
       </c>
@@ -12379,7 +12380,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="127" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A127" s="24">
         <v>166</v>
       </c>
@@ -12448,7 +12449,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="128" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A128" s="24">
         <v>167</v>
       </c>
@@ -12517,7 +12518,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="129" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A129" s="24">
         <v>168</v>
       </c>
@@ -12586,7 +12587,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="130" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A130" s="24">
         <v>169</v>
       </c>
@@ -12655,7 +12656,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="131" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A131" s="24">
         <v>175</v>
       </c>
@@ -12720,7 +12721,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="132" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A132" s="24">
         <v>177</v>
       </c>
@@ -12785,7 +12786,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="133" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A133" s="24">
         <v>178</v>
       </c>
@@ -12850,7 +12851,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="134" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A134" s="24">
         <v>179</v>
       </c>
@@ -12915,7 +12916,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="135" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A135" s="24">
         <v>180</v>
       </c>
@@ -12980,7 +12981,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="136" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A136" s="24">
         <v>181</v>
       </c>
@@ -13045,7 +13046,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="137" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A137" s="24">
         <v>182</v>
       </c>
@@ -13110,7 +13111,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="138" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A138" s="24">
         <v>183</v>
       </c>
@@ -13175,7 +13176,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="139" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A139" s="24">
         <v>184</v>
       </c>
@@ -13240,7 +13241,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="140" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A140" s="24">
         <v>185</v>
       </c>
@@ -13305,7 +13306,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="141" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A141" s="24">
         <v>186</v>
       </c>
@@ -13370,7 +13371,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="142" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A142" s="24">
         <v>187</v>
       </c>
@@ -13435,7 +13436,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="143" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A143" s="24">
         <v>188</v>
       </c>
@@ -13500,7 +13501,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="144" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A144" s="24">
         <v>189</v>
       </c>
@@ -13565,7 +13566,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="145" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A145" s="24">
         <v>190</v>
       </c>
@@ -13658,7 +13659,7 @@
         <v>612</v>
       </c>
       <c r="K146" s="41" t="s">
-        <v>440</v>
+        <v>227</v>
       </c>
       <c r="L146" s="41" t="s">
         <v>440</v>
@@ -13721,7 +13722,7 @@
         <v>612</v>
       </c>
       <c r="K147" s="41" t="s">
-        <v>440</v>
+        <v>227</v>
       </c>
       <c r="L147" s="41" t="s">
         <v>440</v>
@@ -13756,7 +13757,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="148" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A148" s="24">
         <v>417</v>
       </c>
@@ -13825,7 +13826,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="149" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A149" s="24">
         <v>418</v>
       </c>
@@ -13894,7 +13895,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="150" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A150" s="24">
         <v>419</v>
       </c>
@@ -13963,7 +13964,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="151" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A151" s="24">
         <v>423</v>
       </c>
@@ -14032,7 +14033,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="152" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A152" s="24">
         <v>424</v>
       </c>
@@ -14126,7 +14127,7 @@
         <v>440</v>
       </c>
       <c r="J153" s="41" t="s">
-        <v>440</v>
+        <v>62</v>
       </c>
       <c r="K153" s="41" t="s">
         <v>440</v>
@@ -14166,7 +14167,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="154" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A154" s="24">
         <v>432</v>
       </c>
@@ -14235,7 +14236,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="155" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A155" s="24">
         <v>433</v>
       </c>
@@ -14304,7 +14305,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="156" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A156" s="24">
         <v>434</v>
       </c>
@@ -14373,7 +14374,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="157" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A157" s="24">
         <v>435</v>
       </c>
@@ -14442,7 +14443,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="158" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A158" s="24">
         <v>437</v>
       </c>
@@ -14511,7 +14512,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="159" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A159" s="24">
         <v>438</v>
       </c>
@@ -14580,7 +14581,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="160" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A160" s="24">
         <v>440</v>
       </c>
@@ -14649,7 +14650,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="161" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A161" s="24">
         <v>441</v>
       </c>
@@ -14718,7 +14719,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="162" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A162" s="24">
         <v>442</v>
       </c>
@@ -14787,7 +14788,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="163" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A163" s="24">
         <v>443</v>
       </c>
@@ -14856,7 +14857,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="164" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A164" s="24">
         <v>448</v>
       </c>
@@ -14925,7 +14926,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="165" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A165" s="24">
         <v>449</v>
       </c>
@@ -14994,7 +14995,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="166" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A166" s="24">
         <v>450</v>
       </c>
@@ -15063,7 +15064,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="167" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A167" s="24">
         <v>451</v>
       </c>
@@ -15132,7 +15133,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="168" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A168" s="24">
         <v>452</v>
       </c>
@@ -15201,7 +15202,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="169" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A169" s="24">
         <v>454</v>
       </c>
@@ -15266,7 +15267,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="170" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A170" s="24">
         <v>455</v>
       </c>
@@ -15331,7 +15332,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="171" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A171" s="24">
         <v>456</v>
       </c>
@@ -15396,7 +15397,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="172" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A172" s="24">
         <v>457</v>
       </c>
@@ -15461,7 +15462,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="173" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A173" s="24">
         <v>458</v>
       </c>
@@ -15526,7 +15527,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="174" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A174" s="24">
         <v>459</v>
       </c>
@@ -15591,7 +15592,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="175" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A175" s="24">
         <v>460</v>
       </c>
@@ -15660,7 +15661,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="176" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A176" s="24">
         <v>461</v>
       </c>
@@ -15729,7 +15730,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="177" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A177" s="24">
         <v>462</v>
       </c>
@@ -15798,7 +15799,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="178" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A178" s="24">
         <v>463</v>
       </c>
@@ -15863,7 +15864,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="179" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A179" s="24">
         <v>464</v>
       </c>
@@ -15928,7 +15929,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="180" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A180" s="24">
         <v>465</v>
       </c>
@@ -15993,7 +15994,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="181" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A181" s="24">
         <v>466</v>
       </c>
@@ -16062,7 +16063,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="182" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A182" s="24">
         <v>467</v>
       </c>
@@ -16131,7 +16132,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="183" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A183" s="24">
         <v>468</v>
       </c>
@@ -16200,7 +16201,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="184" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A184" s="24">
         <v>469</v>
       </c>
@@ -16265,7 +16266,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="185" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A185" s="24">
         <v>470</v>
       </c>
@@ -16334,7 +16335,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="186" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A186" s="24">
         <v>471</v>
       </c>
@@ -16403,7 +16404,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="187" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A187" s="24">
         <v>472</v>
       </c>
@@ -16472,7 +16473,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="188" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A188" s="24">
         <v>473</v>
       </c>
@@ -16541,7 +16542,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="189" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A189" s="24">
         <v>474</v>
       </c>
@@ -16610,7 +16611,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="190" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A190" s="24">
         <v>475</v>
       </c>
@@ -16679,7 +16680,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="191" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A191" s="24">
         <v>476</v>
       </c>
@@ -16744,7 +16745,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="192" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A192" s="24">
         <v>477</v>
       </c>
@@ -16809,7 +16810,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="193" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A193" s="24">
         <v>478</v>
       </c>
@@ -20826,7 +20827,17 @@
       <c r="W745" s="27"/>
     </row>
   </sheetData>
-  <autoFilter ref="A9:W193" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
+  <autoFilter ref="A9:W193" xr:uid="{00000000-0001-0000-0200-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="191"/>
+        <filter val="376"/>
+        <filter val="425"/>
+        <filter val="47"/>
+        <filter val="48"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="7">
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A2:B2"/>
@@ -23096,12 +23107,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BE9A258ADBC3EC4CBEB1E2AB9909207A" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0284f501378927579289f00316ec8a74">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="295b7897-c886-40bf-9750-5782b814c3e4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b47213d65be806e283915cff374a7eef" ns2:_="">
     <xsd:import namespace="295b7897-c886-40bf-9750-5782b814c3e4"/>
@@ -23245,6 +23250,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -23255,23 +23266,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7568E770-0BC4-46AF-B6C6-958AE21C8F7F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -23289,6 +23283,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Ripetizione test 419, 448, 449, 471 a seguito segnalazione:
Da: fse_support <fse_support@sogei.it> 
Inviato: mercoledì 18 marzo 2026 18:45
A: Simone Ing Bettini | Gas.Net Engineering srl <simone.bettini@gasnet.it>; Sebastiano Bottaro | D.N.A. srl | Gas.Net Group company <sebastiano.bottaro@gasnet.it>
Cc: FSE 2.0 - PNRR <fse-pnrr@innovazione.gov.it>
Oggetto: Mancato accreditamento A1#111#GASNETGROUPXX - gasnet - SaniPocket - V1.0

⚠ Attenzione: messaggio proveniente da un mittente esterno all'organizzazione. 
Diffusione Limitata

Salve,
Con la presente si comunica il mancato superamento dei seguenti test [448, 449, 419, 471] per il servizio [validazione/pubblicazione] del Fornitore [A1#111#GASNETGROUPXX] - Vendor:[gasnet] - ID: [SaniPocket] - Version: [V1.0] - Sha: [56807c0a1dccab32c8633cdb608f4cb372d59585] in data odierna.
Saluti,
Il Team FSE 2.0
________________________________________
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#GASNETGROUPXX/gasnet/SaniPocket/V1.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#GASNETGROUPXX/gasnet/SaniPocket/V1.0/report-checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\simone.bettini\Desktop\temp\20260310_labelling_nazionale_LAB_LDO_RAD_RAP_RSA\SUBMISSION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E245846C-7BDE-4EEB-9A39-C8A7016C6CCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8099B23F-36A3-4AB8-9D48-FAF2CDD9047B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3597" uniqueCount="618">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3597" uniqueCount="616">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -1977,12 +1977,6 @@
     <t>2.16.840.1.113883.2.9.2.50.4.5.50122.a9bce8ce225a9d2a7547e9c1bf9a338f8c11cca0aeb254a12659d7cc82ef526a.e599f7084c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
-    <t>9fcbde8696e5549b85d3f315e3fb4330</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.50.4.5.050234.e5f4f4b379b1c6788d3ec0943e8129437c68075e18abd050c7932c56841ee5da.d5a5d97725^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>777da5d530f417b26c048d746d8c4841</t>
   </si>
   <si>
@@ -2049,18 +2043,6 @@
     <t>2.16.840.1.113883.2.9.2.50.4.5.30345.a54593994ef7b05118b20f6f168055ed4323b46afcc93e057bbd7d4b67748990.63060d7c31^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
-    <t>7d8d9e348070f18e113f1b8ef184804d</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.ce75fa21b4^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>e694e38b7be51f2121b131d4a8a9d1a0</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.ebfff761be^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>4a39f0a78b67dfbd4e784bc7fb815363</t>
   </si>
   <si>
@@ -2121,12 +2103,6 @@
     <t>2.16.840.1.113883.2.9.2.50.4.5.30345.a54593994ef7b05118b20f6f168055ed4323b46afcc93e057bbd7d4b67748990.ee5036df1f^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
-    <t>9f022fc52f16b638c1301e6ae744ed0a</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.50.4.4.2f7f4cb63fd147f6391a5dda313a5b55c1a7f7b94f328efcb0dce010c7118e3d.31d81c9ef9^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>a49f4a815b0b475d41b46e79cd4427e1</t>
   </si>
   <si>
@@ -2167,6 +2143,24 @@
   </si>
   <si>
     <t>GasNet</t>
+  </si>
+  <si>
+    <t>dc79db84bb40ee2ba754b7514c9cc97e</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.641ff8164a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.d8af80d2ab^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>7840b1d8a740d148b45d95f594375f93</t>
+  </si>
+  <si>
+    <t>801f8c38e15d549d4e08f2d194b9dd08</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.50.4.5.50234.e5f4f4b379b1c6788d3ec0943e8129437c68075e18abd050c7932c56841ee5da.e5c5efa562^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -2310,7 +2304,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2327,6 +2321,12 @@
       <patternFill patternType="solid">
         <fgColor theme="4"/>
         <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -2675,7 +2675,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2811,6 +2811,34 @@
     <xf numFmtId="164" fontId="14" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -4279,7 +4307,6 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:W745"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
@@ -4324,14 +4351,14 @@
       <c r="W1" s="30"/>
     </row>
     <row r="2" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="62" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="54" t="s">
-        <v>617</v>
-      </c>
-      <c r="D2" s="55"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="64" t="s">
+        <v>609</v>
+      </c>
+      <c r="D2" s="65"/>
       <c r="F2" s="26"/>
       <c r="G2" s="26"/>
       <c r="H2" s="26"/>
@@ -4352,14 +4379,14 @@
       <c r="W2" s="30"/>
     </row>
     <row r="3" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="66" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="57"/>
-      <c r="C3" s="54" t="s">
-        <v>614</v>
-      </c>
-      <c r="D3" s="55"/>
+      <c r="B3" s="67"/>
+      <c r="C3" s="64" t="s">
+        <v>606</v>
+      </c>
+      <c r="D3" s="65"/>
       <c r="F3" s="26"/>
       <c r="G3" s="26"/>
       <c r="H3" s="26"/>
@@ -4380,12 +4407,12 @@
       <c r="W3" s="30"/>
     </row>
     <row r="4" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="58"/>
-      <c r="B4" s="59"/>
-      <c r="C4" s="54" t="s">
-        <v>615</v>
-      </c>
-      <c r="D4" s="55"/>
+      <c r="A4" s="68"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="64" t="s">
+        <v>607</v>
+      </c>
+      <c r="D4" s="65"/>
       <c r="F4" s="26"/>
       <c r="G4" s="26"/>
       <c r="H4" s="26"/>
@@ -4406,12 +4433,12 @@
       <c r="W4" s="30"/>
     </row>
     <row r="5" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="60"/>
-      <c r="B5" s="61"/>
-      <c r="C5" s="54" t="s">
-        <v>616</v>
-      </c>
-      <c r="D5" s="55"/>
+      <c r="A5" s="70"/>
+      <c r="B5" s="71"/>
+      <c r="C5" s="64" t="s">
+        <v>608</v>
+      </c>
+      <c r="D5" s="65"/>
       <c r="F5" s="26"/>
       <c r="G5" s="26"/>
       <c r="H5" s="26"/>
@@ -4432,8 +4459,8 @@
       <c r="W5" s="30"/>
     </row>
     <row r="6" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="51"/>
-      <c r="B6" s="51"/>
+      <c r="A6" s="61"/>
+      <c r="B6" s="61"/>
       <c r="C6" s="31"/>
       <c r="F6" s="26"/>
       <c r="G6" s="26"/>
@@ -4568,7 +4595,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="36">
         <v>4</v>
       </c>
@@ -4628,7 +4655,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="24">
         <v>28</v>
       </c>
@@ -4684,7 +4711,7 @@
         <v>62</v>
       </c>
       <c r="S11" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T11" s="41"/>
       <c r="U11" s="42" t="s">
@@ -4697,7 +4724,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="24">
         <v>29</v>
       </c>
@@ -4753,7 +4780,7 @@
         <v>62</v>
       </c>
       <c r="S12" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T12" s="41"/>
       <c r="U12" s="42" t="s">
@@ -4766,7 +4793,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="24">
         <v>30</v>
       </c>
@@ -4831,7 +4858,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="24">
         <v>31</v>
       </c>
@@ -4887,7 +4914,7 @@
         <v>62</v>
       </c>
       <c r="S14" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T14" s="41"/>
       <c r="U14" s="42" t="s">
@@ -4900,7 +4927,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="13.5" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="24">
         <v>32</v>
       </c>
@@ -4956,7 +4983,7 @@
         <v>62</v>
       </c>
       <c r="S15" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T15" s="41"/>
       <c r="U15" s="42" t="s">
@@ -4969,7 +4996,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="24">
         <v>33</v>
       </c>
@@ -5034,7 +5061,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="24">
         <v>34</v>
       </c>
@@ -5099,7 +5126,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="24">
         <v>35</v>
       </c>
@@ -5164,7 +5191,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="19" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="24">
         <v>36</v>
       </c>
@@ -5220,7 +5247,7 @@
         <v>62</v>
       </c>
       <c r="S19" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T19" s="41"/>
       <c r="U19" s="42" t="s">
@@ -5233,7 +5260,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="20" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="24">
         <v>37</v>
       </c>
@@ -5289,7 +5316,7 @@
         <v>62</v>
       </c>
       <c r="S20" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T20" s="41"/>
       <c r="U20" s="42" t="s">
@@ -5302,7 +5329,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="24">
         <v>38</v>
       </c>
@@ -5367,7 +5394,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="22" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="24">
         <v>39</v>
       </c>
@@ -5423,7 +5450,7 @@
         <v>62</v>
       </c>
       <c r="S22" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T22" s="41"/>
       <c r="U22" s="42" t="s">
@@ -5436,7 +5463,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="24">
         <v>40</v>
       </c>
@@ -5492,7 +5519,7 @@
         <v>62</v>
       </c>
       <c r="S23" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T23" s="41"/>
       <c r="U23" s="42" t="s">
@@ -5505,7 +5532,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="24" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="24">
         <v>41</v>
       </c>
@@ -5570,7 +5597,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="24">
         <v>42</v>
       </c>
@@ -5635,7 +5662,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="26" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="24">
         <v>43</v>
       </c>
@@ -5700,7 +5727,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="27" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="24">
         <v>44</v>
       </c>
@@ -5752,7 +5779,7 @@
         <v>62</v>
       </c>
       <c r="S27" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T27" s="41"/>
       <c r="U27" s="42" t="s">
@@ -5765,7 +5792,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="28" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="24">
         <v>45</v>
       </c>
@@ -5817,7 +5844,7 @@
         <v>62</v>
       </c>
       <c r="S28" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T28" s="41"/>
       <c r="U28" s="42" t="s">
@@ -5830,7 +5857,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="24">
         <v>46</v>
       </c>
@@ -5947,7 +5974,7 @@
         <v>62</v>
       </c>
       <c r="S30" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T30" s="41"/>
       <c r="U30" s="42" t="s">
@@ -6012,7 +6039,7 @@
         <v>62</v>
       </c>
       <c r="S31" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T31" s="41"/>
       <c r="U31" s="42" t="s">
@@ -6025,7 +6052,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="32" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="24">
         <v>49</v>
       </c>
@@ -6090,7 +6117,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="33" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A33" s="24">
         <v>50</v>
       </c>
@@ -6155,7 +6182,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="34" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34" s="24">
         <v>51</v>
       </c>
@@ -6220,7 +6247,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="35" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A35" s="24">
         <v>53</v>
       </c>
@@ -6276,7 +6303,7 @@
         <v>62</v>
       </c>
       <c r="S35" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T35" s="41"/>
       <c r="U35" s="42" t="s">
@@ -6289,7 +6316,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="36" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="24">
         <v>55</v>
       </c>
@@ -6345,7 +6372,7 @@
         <v>62</v>
       </c>
       <c r="S36" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T36" s="41"/>
       <c r="U36" s="42" t="s">
@@ -6358,7 +6385,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="37" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="24">
         <v>56</v>
       </c>
@@ -6414,7 +6441,7 @@
         <v>62</v>
       </c>
       <c r="S37" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T37" s="41"/>
       <c r="U37" s="42" t="s">
@@ -6427,7 +6454,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="38" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A38" s="24">
         <v>57</v>
       </c>
@@ -6483,7 +6510,7 @@
         <v>62</v>
       </c>
       <c r="S38" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T38" s="41"/>
       <c r="U38" s="42" t="s">
@@ -6496,7 +6523,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="39" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A39" s="24">
         <v>59</v>
       </c>
@@ -6552,7 +6579,7 @@
         <v>62</v>
       </c>
       <c r="S39" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T39" s="41"/>
       <c r="U39" s="42" t="s">
@@ -6565,7 +6592,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="40" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A40" s="24">
         <v>60</v>
       </c>
@@ -6621,7 +6648,7 @@
         <v>62</v>
       </c>
       <c r="S40" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T40" s="41"/>
       <c r="U40" s="42" t="s">
@@ -6634,7 +6661,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="41" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A41" s="24">
         <v>61</v>
       </c>
@@ -6690,7 +6717,7 @@
         <v>62</v>
       </c>
       <c r="S41" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T41" s="41"/>
       <c r="U41" s="42" t="s">
@@ -6703,7 +6730,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="42" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A42" s="24">
         <v>62</v>
       </c>
@@ -6759,7 +6786,7 @@
         <v>62</v>
       </c>
       <c r="S42" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T42" s="41"/>
       <c r="U42" s="42" t="s">
@@ -6772,7 +6799,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="43" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A43" s="24">
         <v>64</v>
       </c>
@@ -6828,7 +6855,7 @@
         <v>62</v>
       </c>
       <c r="S43" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T43" s="41"/>
       <c r="U43" s="42" t="s">
@@ -6841,7 +6868,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="44" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A44" s="24">
         <v>66</v>
       </c>
@@ -6897,7 +6924,7 @@
         <v>62</v>
       </c>
       <c r="S44" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T44" s="41"/>
       <c r="U44" s="42" t="s">
@@ -6910,7 +6937,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A45" s="24">
         <v>67</v>
       </c>
@@ -6966,7 +6993,7 @@
         <v>62</v>
       </c>
       <c r="S45" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T45" s="41"/>
       <c r="U45" s="42" t="s">
@@ -6979,7 +7006,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A46" s="24">
         <v>68</v>
       </c>
@@ -7035,7 +7062,7 @@
         <v>62</v>
       </c>
       <c r="S46" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T46" s="41"/>
       <c r="U46" s="42" t="s">
@@ -7048,7 +7075,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="47" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="24">
         <v>69</v>
       </c>
@@ -7104,7 +7131,7 @@
         <v>62</v>
       </c>
       <c r="S47" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T47" s="41"/>
       <c r="U47" s="42" t="s">
@@ -7117,7 +7144,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="48" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A48" s="24">
         <v>70</v>
       </c>
@@ -7173,7 +7200,7 @@
         <v>62</v>
       </c>
       <c r="S48" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T48" s="41"/>
       <c r="U48" s="42" t="s">
@@ -7186,7 +7213,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="49" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A49" s="24">
         <v>71</v>
       </c>
@@ -7242,7 +7269,7 @@
         <v>62</v>
       </c>
       <c r="S49" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T49" s="41"/>
       <c r="U49" s="42" t="s">
@@ -7255,7 +7282,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="50" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A50" s="24">
         <v>72</v>
       </c>
@@ -7311,7 +7338,7 @@
         <v>62</v>
       </c>
       <c r="S50" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T50" s="41"/>
       <c r="U50" s="42" t="s">
@@ -7324,7 +7351,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="51" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A51" s="24">
         <v>73</v>
       </c>
@@ -7380,7 +7407,7 @@
         <v>62</v>
       </c>
       <c r="S51" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T51" s="41"/>
       <c r="U51" s="42" t="s">
@@ -7393,7 +7420,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="52" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A52" s="24">
         <v>74</v>
       </c>
@@ -7449,7 +7476,7 @@
         <v>62</v>
       </c>
       <c r="S52" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T52" s="41"/>
       <c r="U52" s="42" t="s">
@@ -7462,7 +7489,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="53" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A53" s="24">
         <v>76</v>
       </c>
@@ -7518,7 +7545,7 @@
         <v>62</v>
       </c>
       <c r="S53" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T53" s="41"/>
       <c r="U53" s="42" t="s">
@@ -7531,7 +7558,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="54" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="24">
         <v>78</v>
       </c>
@@ -7587,7 +7614,7 @@
         <v>62</v>
       </c>
       <c r="S54" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T54" s="41"/>
       <c r="U54" s="42" t="s">
@@ -7600,7 +7627,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="55" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A55" s="24">
         <v>79</v>
       </c>
@@ -7656,7 +7683,7 @@
         <v>62</v>
       </c>
       <c r="S55" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T55" s="41"/>
       <c r="U55" s="42" t="s">
@@ -7669,7 +7696,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="56" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A56" s="24">
         <v>80</v>
       </c>
@@ -7725,7 +7752,7 @@
         <v>62</v>
       </c>
       <c r="S56" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T56" s="41"/>
       <c r="U56" s="42" t="s">
@@ -7738,7 +7765,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="57" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A57" s="24">
         <v>81</v>
       </c>
@@ -7794,7 +7821,7 @@
         <v>62</v>
       </c>
       <c r="S57" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T57" s="41"/>
       <c r="U57" s="42" t="s">
@@ -7807,7 +7834,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="58" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A58" s="24">
         <v>83</v>
       </c>
@@ -7863,7 +7890,7 @@
         <v>62</v>
       </c>
       <c r="S58" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T58" s="41"/>
       <c r="U58" s="42" t="s">
@@ -7876,7 +7903,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="59" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A59" s="24">
         <v>84</v>
       </c>
@@ -7932,7 +7959,7 @@
         <v>62</v>
       </c>
       <c r="S59" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T59" s="41"/>
       <c r="U59" s="42" t="s">
@@ -7945,7 +7972,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="60" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A60" s="24">
         <v>85</v>
       </c>
@@ -8001,7 +8028,7 @@
         <v>62</v>
       </c>
       <c r="S60" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T60" s="41"/>
       <c r="U60" s="42" t="s">
@@ -8014,7 +8041,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="61" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A61" s="24">
         <v>86</v>
       </c>
@@ -8070,7 +8097,7 @@
         <v>62</v>
       </c>
       <c r="S61" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T61" s="41"/>
       <c r="U61" s="42" t="s">
@@ -8083,7 +8110,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="62" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A62" s="24">
         <v>87</v>
       </c>
@@ -8139,7 +8166,7 @@
         <v>62</v>
       </c>
       <c r="S62" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T62" s="41"/>
       <c r="U62" s="42" t="s">
@@ -8152,7 +8179,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="63" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A63" s="24">
         <v>88</v>
       </c>
@@ -8208,7 +8235,7 @@
         <v>62</v>
       </c>
       <c r="S63" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T63" s="41"/>
       <c r="U63" s="42" t="s">
@@ -8221,7 +8248,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="64" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A64" s="24">
         <v>89</v>
       </c>
@@ -8277,7 +8304,7 @@
         <v>62</v>
       </c>
       <c r="S64" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T64" s="41"/>
       <c r="U64" s="42" t="s">
@@ -8290,7 +8317,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="65" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A65" s="24">
         <v>90</v>
       </c>
@@ -8346,7 +8373,7 @@
         <v>62</v>
       </c>
       <c r="S65" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T65" s="41"/>
       <c r="U65" s="42" t="s">
@@ -8359,7 +8386,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="66" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A66" s="24">
         <v>91</v>
       </c>
@@ -8415,7 +8442,7 @@
         <v>62</v>
       </c>
       <c r="S66" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T66" s="41"/>
       <c r="U66" s="42" t="s">
@@ -8428,7 +8455,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="67" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A67" s="24">
         <v>92</v>
       </c>
@@ -8484,7 +8511,7 @@
         <v>62</v>
       </c>
       <c r="S67" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T67" s="41"/>
       <c r="U67" s="42" t="s">
@@ -8497,7 +8524,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="68" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A68" s="24">
         <v>93</v>
       </c>
@@ -8553,7 +8580,7 @@
         <v>62</v>
       </c>
       <c r="S68" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T68" s="41"/>
       <c r="U68" s="42" t="s">
@@ -8566,7 +8593,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="69" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A69" s="24">
         <v>95</v>
       </c>
@@ -8631,7 +8658,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="70" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A70" s="24">
         <v>97</v>
       </c>
@@ -8696,7 +8723,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="71" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A71" s="24">
         <v>98</v>
       </c>
@@ -8761,7 +8788,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="72" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A72" s="24">
         <v>99</v>
       </c>
@@ -8826,7 +8853,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="73" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A73" s="24">
         <v>100</v>
       </c>
@@ -8891,7 +8918,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="74" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A74" s="24">
         <v>101</v>
       </c>
@@ -8956,7 +8983,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="75" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A75" s="24">
         <v>102</v>
       </c>
@@ -9021,7 +9048,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="76" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A76" s="24">
         <v>103</v>
       </c>
@@ -9086,7 +9113,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="77" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A77" s="24">
         <v>104</v>
       </c>
@@ -9151,7 +9178,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="78" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A78" s="24">
         <v>105</v>
       </c>
@@ -9216,7 +9243,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="79" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A79" s="24">
         <v>106</v>
       </c>
@@ -9281,7 +9308,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="80" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A80" s="24">
         <v>108</v>
       </c>
@@ -9346,7 +9373,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="81" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A81" s="24">
         <v>110</v>
       </c>
@@ -9411,7 +9438,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="82" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A82" s="24">
         <v>111</v>
       </c>
@@ -9476,7 +9503,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="83" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A83" s="24">
         <v>112</v>
       </c>
@@ -9541,7 +9568,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="84" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A84" s="24">
         <v>113</v>
       </c>
@@ -9606,7 +9633,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="85" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A85" s="24">
         <v>114</v>
       </c>
@@ -9671,7 +9698,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="86" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A86" s="24">
         <v>115</v>
       </c>
@@ -9736,7 +9763,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="87" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A87" s="24">
         <v>116</v>
       </c>
@@ -9801,7 +9828,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="88" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A88" s="24">
         <v>117</v>
       </c>
@@ -9866,7 +9893,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="89" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A89" s="24">
         <v>118</v>
       </c>
@@ -9931,7 +9958,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="90" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A90" s="24">
         <v>119</v>
       </c>
@@ -9996,7 +10023,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="91" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A91" s="24">
         <v>120</v>
       </c>
@@ -10061,7 +10088,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="92" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A92" s="24">
         <v>121</v>
       </c>
@@ -10126,7 +10153,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="93" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A93" s="24">
         <v>123</v>
       </c>
@@ -10191,7 +10218,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="94" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A94" s="24">
         <v>125</v>
       </c>
@@ -10256,7 +10283,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="95" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A95" s="24">
         <v>126</v>
       </c>
@@ -10321,7 +10348,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="96" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A96" s="24">
         <v>127</v>
       </c>
@@ -10386,7 +10413,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="97" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A97" s="24">
         <v>128</v>
       </c>
@@ -10451,7 +10478,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="98" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A98" s="24">
         <v>129</v>
       </c>
@@ -10516,7 +10543,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="99" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A99" s="24">
         <v>130</v>
       </c>
@@ -10581,7 +10608,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="100" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A100" s="24">
         <v>131</v>
       </c>
@@ -10646,7 +10673,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="101" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A101" s="24">
         <v>132</v>
       </c>
@@ -10711,7 +10738,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="102" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A102" s="24">
         <v>133</v>
       </c>
@@ -10776,7 +10803,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="103" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A103" s="24">
         <v>134</v>
       </c>
@@ -10841,7 +10868,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="104" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A104" s="24">
         <v>135</v>
       </c>
@@ -10906,7 +10933,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="105" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A105" s="24">
         <v>136</v>
       </c>
@@ -10971,7 +10998,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="106" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A106" s="24">
         <v>137</v>
       </c>
@@ -11036,7 +11063,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="107" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A107" s="24">
         <v>138</v>
       </c>
@@ -11101,7 +11128,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="108" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A108" s="24">
         <v>139</v>
       </c>
@@ -11166,7 +11193,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="109" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A109" s="24">
         <v>140</v>
       </c>
@@ -11231,7 +11258,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="110" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A110" s="24">
         <v>141</v>
       </c>
@@ -11296,7 +11323,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="111" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A111" s="24">
         <v>142</v>
       </c>
@@ -11361,7 +11388,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="112" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A112" s="24">
         <v>143</v>
       </c>
@@ -11426,7 +11453,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="113" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A113" s="24">
         <v>144</v>
       </c>
@@ -11491,7 +11518,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="114" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A114" s="24">
         <v>145</v>
       </c>
@@ -11556,7 +11583,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="115" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A115" s="24">
         <v>146</v>
       </c>
@@ -11621,7 +11648,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="116" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A116" s="24">
         <v>152</v>
       </c>
@@ -11677,7 +11704,7 @@
         <v>62</v>
       </c>
       <c r="S116" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T116" s="41"/>
       <c r="U116" s="42" t="s">
@@ -11690,7 +11717,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="117" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A117" s="24">
         <v>154</v>
       </c>
@@ -11746,7 +11773,7 @@
         <v>62</v>
       </c>
       <c r="S117" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T117" s="41"/>
       <c r="U117" s="42" t="s">
@@ -11759,7 +11786,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="118" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A118" s="24">
         <v>155</v>
       </c>
@@ -11815,7 +11842,7 @@
         <v>62</v>
       </c>
       <c r="S118" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T118" s="41"/>
       <c r="U118" s="42" t="s">
@@ -11828,7 +11855,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="119" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A119" s="24">
         <v>156</v>
       </c>
@@ -11884,7 +11911,7 @@
         <v>62</v>
       </c>
       <c r="S119" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T119" s="41"/>
       <c r="U119" s="42" t="s">
@@ -11897,7 +11924,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="120" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A120" s="24">
         <v>159</v>
       </c>
@@ -11953,7 +11980,7 @@
         <v>62</v>
       </c>
       <c r="S120" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T120" s="41"/>
       <c r="U120" s="42" t="s">
@@ -11966,7 +11993,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="121" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A121" s="24">
         <v>160</v>
       </c>
@@ -12022,7 +12049,7 @@
         <v>62</v>
       </c>
       <c r="S121" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T121" s="41"/>
       <c r="U121" s="42" t="s">
@@ -12035,7 +12062,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="122" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A122" s="24">
         <v>161</v>
       </c>
@@ -12091,7 +12118,7 @@
         <v>62</v>
       </c>
       <c r="S122" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T122" s="41"/>
       <c r="U122" s="42" t="s">
@@ -12104,7 +12131,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="123" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A123" s="24">
         <v>162</v>
       </c>
@@ -12160,7 +12187,7 @@
         <v>62</v>
       </c>
       <c r="S123" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T123" s="41"/>
       <c r="U123" s="42" t="s">
@@ -12173,7 +12200,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="124" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A124" s="24">
         <v>163</v>
       </c>
@@ -12229,7 +12256,7 @@
         <v>62</v>
       </c>
       <c r="S124" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T124" s="41"/>
       <c r="U124" s="42" t="s">
@@ -12242,7 +12269,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="125" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A125" s="24">
         <v>164</v>
       </c>
@@ -12298,7 +12325,7 @@
         <v>62</v>
       </c>
       <c r="S125" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T125" s="41"/>
       <c r="U125" s="42" t="s">
@@ -12311,7 +12338,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="126" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A126" s="24">
         <v>165</v>
       </c>
@@ -12367,7 +12394,7 @@
         <v>62</v>
       </c>
       <c r="S126" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T126" s="41"/>
       <c r="U126" s="42" t="s">
@@ -12380,7 +12407,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="127" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A127" s="24">
         <v>166</v>
       </c>
@@ -12436,7 +12463,7 @@
         <v>62</v>
       </c>
       <c r="S127" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T127" s="41"/>
       <c r="U127" s="42" t="s">
@@ -12449,7 +12476,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="128" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A128" s="24">
         <v>167</v>
       </c>
@@ -12505,7 +12532,7 @@
         <v>62</v>
       </c>
       <c r="S128" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T128" s="41"/>
       <c r="U128" s="42" t="s">
@@ -12518,7 +12545,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="129" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A129" s="24">
         <v>168</v>
       </c>
@@ -12574,7 +12601,7 @@
         <v>62</v>
       </c>
       <c r="S129" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T129" s="41"/>
       <c r="U129" s="42" t="s">
@@ -12587,7 +12614,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="130" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A130" s="24">
         <v>169</v>
       </c>
@@ -12643,7 +12670,7 @@
         <v>62</v>
       </c>
       <c r="S130" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T130" s="41"/>
       <c r="U130" s="42" t="s">
@@ -12656,7 +12683,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="131" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A131" s="24">
         <v>175</v>
       </c>
@@ -12721,7 +12748,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="132" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A132" s="24">
         <v>177</v>
       </c>
@@ -12786,7 +12813,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="133" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A133" s="24">
         <v>178</v>
       </c>
@@ -12851,7 +12878,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="134" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A134" s="24">
         <v>179</v>
       </c>
@@ -12916,7 +12943,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="135" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A135" s="24">
         <v>180</v>
       </c>
@@ -12981,7 +13008,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="136" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A136" s="24">
         <v>181</v>
       </c>
@@ -13046,7 +13073,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="137" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A137" s="24">
         <v>182</v>
       </c>
@@ -13111,7 +13138,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="138" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A138" s="24">
         <v>183</v>
       </c>
@@ -13176,7 +13203,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="139" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A139" s="24">
         <v>184</v>
       </c>
@@ -13241,7 +13268,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="140" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A140" s="24">
         <v>185</v>
       </c>
@@ -13306,7 +13333,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="141" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A141" s="24">
         <v>186</v>
       </c>
@@ -13371,7 +13398,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="142" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A142" s="24">
         <v>187</v>
       </c>
@@ -13436,7 +13463,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="143" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A143" s="24">
         <v>188</v>
       </c>
@@ -13501,7 +13528,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="144" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A144" s="24">
         <v>189</v>
       </c>
@@ -13566,7 +13593,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="145" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A145" s="24">
         <v>190</v>
       </c>
@@ -13656,7 +13683,7 @@
         <v>440</v>
       </c>
       <c r="J146" s="41" t="s">
-        <v>612</v>
+        <v>604</v>
       </c>
       <c r="K146" s="41" t="s">
         <v>227</v>
@@ -13719,7 +13746,7 @@
         <v>440</v>
       </c>
       <c r="J147" s="41" t="s">
-        <v>612</v>
+        <v>604</v>
       </c>
       <c r="K147" s="41" t="s">
         <v>227</v>
@@ -13757,7 +13784,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="148" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A148" s="24">
         <v>417</v>
       </c>
@@ -13813,7 +13840,7 @@
         <v>62</v>
       </c>
       <c r="S148" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T148" s="41"/>
       <c r="U148" s="42" t="s">
@@ -13826,7 +13853,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="149" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A149" s="24">
         <v>418</v>
       </c>
@@ -13882,7 +13909,7 @@
         <v>62</v>
       </c>
       <c r="S149" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T149" s="41"/>
       <c r="U149" s="42" t="s">
@@ -13895,76 +13922,76 @@
         <v>36</v>
       </c>
     </row>
-    <row r="150" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A150" s="24">
+    <row r="150" spans="1:23" s="60" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A150" s="51">
         <v>419</v>
       </c>
-      <c r="B150" s="24" t="s">
+      <c r="B150" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="C150" s="44" t="s">
+      <c r="C150" s="52" t="s">
         <v>239</v>
       </c>
-      <c r="D150" s="24" t="s">
+      <c r="D150" s="51" t="s">
         <v>242</v>
       </c>
-      <c r="E150" s="38" t="s">
+      <c r="E150" s="53" t="s">
         <v>267</v>
       </c>
-      <c r="F150" s="40">
+      <c r="F150" s="54">
         <v>46090</v>
       </c>
-      <c r="G150" s="40">
-        <v>46090.528356481482</v>
-      </c>
-      <c r="H150" s="40" t="s">
-        <v>554</v>
-      </c>
-      <c r="I150" s="50" t="s">
-        <v>555</v>
-      </c>
-      <c r="J150" s="41" t="s">
+      <c r="G150" s="54">
+        <v>46100.38175925926</v>
+      </c>
+      <c r="H150" s="54" t="s">
+        <v>614</v>
+      </c>
+      <c r="I150" s="55" t="s">
+        <v>615</v>
+      </c>
+      <c r="J150" s="56" t="s">
         <v>439</v>
       </c>
-      <c r="K150" s="41" t="s">
-        <v>440</v>
-      </c>
-      <c r="L150" s="41" t="s">
-        <v>440</v>
-      </c>
-      <c r="M150" s="41" t="s">
-        <v>224</v>
-      </c>
-      <c r="N150" s="41" t="s">
-        <v>224</v>
-      </c>
-      <c r="O150" s="41" t="s">
-        <v>440</v>
-      </c>
-      <c r="P150" s="41" t="s">
+      <c r="K150" s="56" t="s">
+        <v>440</v>
+      </c>
+      <c r="L150" s="56" t="s">
+        <v>440</v>
+      </c>
+      <c r="M150" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="N150" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="O150" s="56" t="s">
+        <v>440</v>
+      </c>
+      <c r="P150" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="Q150" s="41" t="s">
-        <v>224</v>
-      </c>
-      <c r="R150" s="41" t="s">
+      <c r="Q150" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="R150" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="S150" s="46" t="s">
-        <v>613</v>
-      </c>
-      <c r="T150" s="41"/>
-      <c r="U150" s="42" t="s">
-        <v>440</v>
-      </c>
-      <c r="V150" s="43" t="s">
-        <v>440</v>
-      </c>
-      <c r="W150" s="41" t="s">
+      <c r="S150" s="57" t="s">
+        <v>605</v>
+      </c>
+      <c r="T150" s="56"/>
+      <c r="U150" s="58" t="s">
+        <v>440</v>
+      </c>
+      <c r="V150" s="59" t="s">
+        <v>440</v>
+      </c>
+      <c r="W150" s="56" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="151" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A151" s="24">
         <v>423</v>
       </c>
@@ -13987,7 +14014,7 @@
         <v>46090.722210648149</v>
       </c>
       <c r="H151" s="40" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="I151" s="50" t="s">
         <v>443</v>
@@ -14020,7 +14047,7 @@
         <v>62</v>
       </c>
       <c r="S151" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T151" s="41"/>
       <c r="U151" s="42" t="s">
@@ -14033,7 +14060,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="152" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A152" s="24">
         <v>424</v>
       </c>
@@ -14056,7 +14083,7 @@
         <v>46090.721863425926</v>
       </c>
       <c r="H152" s="40" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="I152" s="50" t="s">
         <v>443</v>
@@ -14089,7 +14116,7 @@
         <v>62</v>
       </c>
       <c r="S152" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T152" s="41"/>
       <c r="U152" s="42" t="s">
@@ -14154,7 +14181,7 @@
         <v>62</v>
       </c>
       <c r="S153" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T153" s="41"/>
       <c r="U153" s="42" t="s">
@@ -14167,7 +14194,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="154" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A154" s="24">
         <v>432</v>
       </c>
@@ -14190,10 +14217,10 @@
         <v>46090.59003472222</v>
       </c>
       <c r="H154" s="40" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="I154" s="50" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="J154" s="41" t="s">
         <v>439</v>
@@ -14223,7 +14250,7 @@
         <v>62</v>
       </c>
       <c r="S154" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T154" s="41"/>
       <c r="U154" s="42" t="s">
@@ -14236,7 +14263,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="155" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A155" s="24">
         <v>433</v>
       </c>
@@ -14259,10 +14286,10 @@
         <v>46090.590416666666</v>
       </c>
       <c r="H155" s="40" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="I155" s="50" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="J155" s="41" t="s">
         <v>439</v>
@@ -14292,7 +14319,7 @@
         <v>62</v>
       </c>
       <c r="S155" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T155" s="41"/>
       <c r="U155" s="42" t="s">
@@ -14305,7 +14332,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="156" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A156" s="24">
         <v>434</v>
       </c>
@@ -14328,10 +14355,10 @@
         <v>46090.591111111113</v>
       </c>
       <c r="H156" s="40" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="I156" s="50" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="J156" s="41" t="s">
         <v>439</v>
@@ -14361,7 +14388,7 @@
         <v>62</v>
       </c>
       <c r="S156" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T156" s="41"/>
       <c r="U156" s="42" t="s">
@@ -14374,7 +14401,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="157" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A157" s="24">
         <v>435</v>
       </c>
@@ -14397,10 +14424,10 @@
         <v>46090.593935185185</v>
       </c>
       <c r="H157" s="40" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="I157" s="50" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="J157" s="41" t="s">
         <v>439</v>
@@ -14430,7 +14457,7 @@
         <v>62</v>
       </c>
       <c r="S157" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T157" s="41"/>
       <c r="U157" s="42" t="s">
@@ -14443,7 +14470,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="158" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A158" s="24">
         <v>437</v>
       </c>
@@ -14466,10 +14493,10 @@
         <v>46090.594456018516</v>
       </c>
       <c r="H158" s="40" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="I158" s="50" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="J158" s="41" t="s">
         <v>439</v>
@@ -14499,7 +14526,7 @@
         <v>62</v>
       </c>
       <c r="S158" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T158" s="41"/>
       <c r="U158" s="42" t="s">
@@ -14512,7 +14539,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="159" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A159" s="24">
         <v>438</v>
       </c>
@@ -14535,10 +14562,10 @@
         <v>46090.594849537039</v>
       </c>
       <c r="H159" s="40" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="I159" s="50" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="J159" s="41" t="s">
         <v>439</v>
@@ -14568,7 +14595,7 @@
         <v>62</v>
       </c>
       <c r="S159" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T159" s="41"/>
       <c r="U159" s="42" t="s">
@@ -14581,7 +14608,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="160" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A160" s="24">
         <v>440</v>
       </c>
@@ -14604,10 +14631,10 @@
         <v>46090.595138888886</v>
       </c>
       <c r="H160" s="40" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="I160" s="50" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="J160" s="41" t="s">
         <v>439</v>
@@ -14637,7 +14664,7 @@
         <v>62</v>
       </c>
       <c r="S160" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T160" s="41"/>
       <c r="U160" s="42" t="s">
@@ -14650,7 +14677,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="161" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A161" s="24">
         <v>441</v>
       </c>
@@ -14673,10 +14700,10 @@
         <v>46090.595370370371</v>
       </c>
       <c r="H161" s="40" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="I161" s="50" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="J161" s="41" t="s">
         <v>439</v>
@@ -14706,7 +14733,7 @@
         <v>62</v>
       </c>
       <c r="S161" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T161" s="41"/>
       <c r="U161" s="42" t="s">
@@ -14719,7 +14746,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="162" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A162" s="24">
         <v>442</v>
       </c>
@@ -14742,10 +14769,10 @@
         <v>46090.595706018517</v>
       </c>
       <c r="H162" s="40" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="I162" s="50" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="J162" s="41" t="s">
         <v>439</v>
@@ -14775,7 +14802,7 @@
         <v>62</v>
       </c>
       <c r="S162" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T162" s="41"/>
       <c r="U162" s="42" t="s">
@@ -14788,7 +14815,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="163" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A163" s="24">
         <v>443</v>
       </c>
@@ -14811,10 +14838,10 @@
         <v>46090.595902777779</v>
       </c>
       <c r="H163" s="40" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="I163" s="50" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="J163" s="41" t="s">
         <v>439</v>
@@ -14844,7 +14871,7 @@
         <v>62</v>
       </c>
       <c r="S163" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T163" s="41"/>
       <c r="U163" s="42" t="s">
@@ -14857,145 +14884,145 @@
         <v>43</v>
       </c>
     </row>
-    <row r="164" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A164" s="24">
+    <row r="164" spans="1:23" s="60" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="51">
         <v>448</v>
       </c>
-      <c r="B164" s="24" t="s">
+      <c r="B164" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="C164" s="44" t="s">
+      <c r="C164" s="52" t="s">
         <v>48</v>
       </c>
-      <c r="D164" s="24" t="s">
+      <c r="D164" s="51" t="s">
         <v>375</v>
       </c>
-      <c r="E164" s="38" t="s">
+      <c r="E164" s="53" t="s">
         <v>377</v>
       </c>
-      <c r="F164" s="40">
+      <c r="F164" s="54">
         <v>46090</v>
       </c>
-      <c r="G164" s="40">
-        <v>46090.410636574074</v>
-      </c>
-      <c r="H164" s="40" t="s">
-        <v>578</v>
-      </c>
-      <c r="I164" s="50" t="s">
-        <v>579</v>
-      </c>
-      <c r="J164" s="41" t="s">
+      <c r="G164" s="54">
+        <v>46100</v>
+      </c>
+      <c r="H164" s="54" t="s">
+        <v>610</v>
+      </c>
+      <c r="I164" s="55" t="s">
+        <v>612</v>
+      </c>
+      <c r="J164" s="56" t="s">
         <v>439</v>
       </c>
-      <c r="K164" s="41" t="s">
-        <v>440</v>
-      </c>
-      <c r="L164" s="41" t="s">
-        <v>440</v>
-      </c>
-      <c r="M164" s="41" t="s">
-        <v>224</v>
-      </c>
-      <c r="N164" s="41" t="s">
-        <v>224</v>
-      </c>
-      <c r="O164" s="41" t="s">
-        <v>440</v>
-      </c>
-      <c r="P164" s="41" t="s">
+      <c r="K164" s="56" t="s">
+        <v>440</v>
+      </c>
+      <c r="L164" s="56" t="s">
+        <v>440</v>
+      </c>
+      <c r="M164" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="N164" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="O164" s="56" t="s">
+        <v>440</v>
+      </c>
+      <c r="P164" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="Q164" s="41" t="s">
-        <v>224</v>
-      </c>
-      <c r="R164" s="41" t="s">
+      <c r="Q164" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="R164" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="S164" s="46" t="s">
+      <c r="S164" s="57" t="s">
+        <v>605</v>
+      </c>
+      <c r="T164" s="56"/>
+      <c r="U164" s="58" t="s">
+        <v>440</v>
+      </c>
+      <c r="V164" s="59" t="s">
+        <v>440</v>
+      </c>
+      <c r="W164" s="56" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="165" spans="1:23" s="60" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A165" s="51">
+        <v>449</v>
+      </c>
+      <c r="B165" s="51" t="s">
+        <v>34</v>
+      </c>
+      <c r="C165" s="52" t="s">
+        <v>48</v>
+      </c>
+      <c r="D165" s="51" t="s">
+        <v>376</v>
+      </c>
+      <c r="E165" s="53" t="s">
+        <v>378</v>
+      </c>
+      <c r="F165" s="54">
+        <v>46090</v>
+      </c>
+      <c r="G165" s="54">
+        <v>46100</v>
+      </c>
+      <c r="H165" s="54" t="s">
         <v>613</v>
       </c>
-      <c r="T164" s="41"/>
-      <c r="U164" s="42" t="s">
-        <v>440</v>
-      </c>
-      <c r="V164" s="43" t="s">
-        <v>440</v>
-      </c>
-      <c r="W164" s="41" t="s">
+      <c r="I165" s="55" t="s">
+        <v>611</v>
+      </c>
+      <c r="J165" s="56" t="s">
+        <v>439</v>
+      </c>
+      <c r="K165" s="56" t="s">
+        <v>440</v>
+      </c>
+      <c r="L165" s="56" t="s">
+        <v>440</v>
+      </c>
+      <c r="M165" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="N165" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="O165" s="56" t="s">
+        <v>440</v>
+      </c>
+      <c r="P165" s="56" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q165" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="R165" s="56" t="s">
+        <v>62</v>
+      </c>
+      <c r="S165" s="57" t="s">
+        <v>605</v>
+      </c>
+      <c r="T165" s="56"/>
+      <c r="U165" s="58" t="s">
+        <v>440</v>
+      </c>
+      <c r="V165" s="59" t="s">
+        <v>440</v>
+      </c>
+      <c r="W165" s="56" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="165" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A165" s="24">
-        <v>449</v>
-      </c>
-      <c r="B165" s="24" t="s">
-        <v>34</v>
-      </c>
-      <c r="C165" s="44" t="s">
-        <v>48</v>
-      </c>
-      <c r="D165" s="24" t="s">
-        <v>376</v>
-      </c>
-      <c r="E165" s="38" t="s">
-        <v>378</v>
-      </c>
-      <c r="F165" s="40">
-        <v>46090</v>
-      </c>
-      <c r="G165" s="40">
-        <v>46090.41064814815</v>
-      </c>
-      <c r="H165" s="40" t="s">
-        <v>580</v>
-      </c>
-      <c r="I165" s="50" t="s">
-        <v>581</v>
-      </c>
-      <c r="J165" s="41" t="s">
-        <v>439</v>
-      </c>
-      <c r="K165" s="41" t="s">
-        <v>440</v>
-      </c>
-      <c r="L165" s="41" t="s">
-        <v>440</v>
-      </c>
-      <c r="M165" s="41" t="s">
-        <v>224</v>
-      </c>
-      <c r="N165" s="41" t="s">
-        <v>224</v>
-      </c>
-      <c r="O165" s="41" t="s">
-        <v>440</v>
-      </c>
-      <c r="P165" s="41" t="s">
-        <v>62</v>
-      </c>
-      <c r="Q165" s="41" t="s">
-        <v>224</v>
-      </c>
-      <c r="R165" s="41" t="s">
-        <v>62</v>
-      </c>
-      <c r="S165" s="46" t="s">
-        <v>613</v>
-      </c>
-      <c r="T165" s="41"/>
-      <c r="U165" s="42" t="s">
-        <v>440</v>
-      </c>
-      <c r="V165" s="43" t="s">
-        <v>440</v>
-      </c>
-      <c r="W165" s="41" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="166" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A166" s="24">
         <v>450</v>
       </c>
@@ -15018,10 +15045,10 @@
         <v>46090.452824074076</v>
       </c>
       <c r="H166" s="40" t="s">
-        <v>582</v>
+        <v>576</v>
       </c>
       <c r="I166" s="50" t="s">
-        <v>583</v>
+        <v>577</v>
       </c>
       <c r="J166" s="41" t="s">
         <v>439</v>
@@ -15051,7 +15078,7 @@
         <v>62</v>
       </c>
       <c r="S166" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T166" s="41"/>
       <c r="U166" s="42" t="s">
@@ -15064,7 +15091,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="167" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A167" s="24">
         <v>451</v>
       </c>
@@ -15087,10 +15114,10 @@
         <v>46090.452835648146</v>
       </c>
       <c r="H167" s="40" t="s">
-        <v>584</v>
+        <v>578</v>
       </c>
       <c r="I167" s="50" t="s">
-        <v>585</v>
+        <v>579</v>
       </c>
       <c r="J167" s="41" t="s">
         <v>439</v>
@@ -15120,7 +15147,7 @@
         <v>62</v>
       </c>
       <c r="S167" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T167" s="41"/>
       <c r="U167" s="42" t="s">
@@ -15133,7 +15160,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="168" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A168" s="24">
         <v>452</v>
       </c>
@@ -15156,10 +15183,10 @@
         <v>46090.439282407409</v>
       </c>
       <c r="H168" s="40" t="s">
-        <v>586</v>
+        <v>580</v>
       </c>
       <c r="I168" s="50" t="s">
-        <v>587</v>
+        <v>581</v>
       </c>
       <c r="J168" s="41" t="s">
         <v>439</v>
@@ -15189,7 +15216,7 @@
         <v>62</v>
       </c>
       <c r="S168" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T168" s="41"/>
       <c r="U168" s="42" t="s">
@@ -15202,7 +15229,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="169" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A169" s="24">
         <v>454</v>
       </c>
@@ -15267,7 +15294,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="170" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A170" s="24">
         <v>455</v>
       </c>
@@ -15332,7 +15359,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="171" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A171" s="24">
         <v>456</v>
       </c>
@@ -15397,7 +15424,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="172" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A172" s="24">
         <v>457</v>
       </c>
@@ -15462,7 +15489,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="173" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A173" s="24">
         <v>458</v>
       </c>
@@ -15527,7 +15554,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="174" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A174" s="24">
         <v>459</v>
       </c>
@@ -15592,7 +15619,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="175" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A175" s="24">
         <v>460</v>
       </c>
@@ -15615,10 +15642,10 @@
         <v>46090.545011574075</v>
       </c>
       <c r="H175" s="40" t="s">
-        <v>588</v>
+        <v>582</v>
       </c>
       <c r="I175" s="50" t="s">
-        <v>589</v>
+        <v>583</v>
       </c>
       <c r="J175" s="41" t="s">
         <v>439</v>
@@ -15648,7 +15675,7 @@
         <v>62</v>
       </c>
       <c r="S175" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T175" s="41"/>
       <c r="U175" s="42" t="s">
@@ -15661,7 +15688,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="176" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A176" s="24">
         <v>461</v>
       </c>
@@ -15684,10 +15711,10 @@
         <v>46090.41065972222</v>
       </c>
       <c r="H176" s="24" t="s">
-        <v>590</v>
+        <v>584</v>
       </c>
       <c r="I176" s="24" t="s">
-        <v>591</v>
+        <v>585</v>
       </c>
       <c r="J176" s="41" t="s">
         <v>439</v>
@@ -15717,7 +15744,7 @@
         <v>62</v>
       </c>
       <c r="S176" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T176" s="41"/>
       <c r="U176" s="24" t="s">
@@ -15730,7 +15757,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="177" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A177" s="24">
         <v>462</v>
       </c>
@@ -15753,10 +15780,10 @@
         <v>46090.479791666665</v>
       </c>
       <c r="H177" s="24" t="s">
-        <v>592</v>
+        <v>586</v>
       </c>
       <c r="I177" s="24" t="s">
-        <v>593</v>
+        <v>587</v>
       </c>
       <c r="J177" s="41" t="s">
         <v>439</v>
@@ -15786,7 +15813,7 @@
         <v>62</v>
       </c>
       <c r="S177" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T177" s="41"/>
       <c r="U177" s="24" t="s">
@@ -15799,7 +15826,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="178" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A178" s="24">
         <v>463</v>
       </c>
@@ -15864,7 +15891,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="179" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A179" s="24">
         <v>464</v>
       </c>
@@ -15929,7 +15956,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="180" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A180" s="24">
         <v>465</v>
       </c>
@@ -15994,7 +16021,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="181" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A181" s="24">
         <v>466</v>
       </c>
@@ -16017,10 +16044,10 @@
         <v>46090.439293981479</v>
       </c>
       <c r="H181" s="24" t="s">
-        <v>594</v>
+        <v>588</v>
       </c>
       <c r="I181" s="24" t="s">
-        <v>595</v>
+        <v>589</v>
       </c>
       <c r="J181" s="41" t="s">
         <v>439</v>
@@ -16050,7 +16077,7 @@
         <v>62</v>
       </c>
       <c r="S181" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T181" s="41"/>
       <c r="U181" s="24" t="s">
@@ -16063,7 +16090,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="182" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A182" s="24">
         <v>467</v>
       </c>
@@ -16086,10 +16113,10 @@
         <v>46090.452835648146</v>
       </c>
       <c r="H182" s="24" t="s">
-        <v>596</v>
+        <v>590</v>
       </c>
       <c r="I182" s="24" t="s">
-        <v>597</v>
+        <v>591</v>
       </c>
       <c r="J182" s="41" t="s">
         <v>439</v>
@@ -16119,7 +16146,7 @@
         <v>62</v>
       </c>
       <c r="S182" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T182" s="41"/>
       <c r="U182" s="24" t="s">
@@ -16132,7 +16159,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="183" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A183" s="24">
         <v>468</v>
       </c>
@@ -16155,10 +16182,10 @@
         <v>46090.41065972222</v>
       </c>
       <c r="H183" s="24" t="s">
-        <v>598</v>
+        <v>592</v>
       </c>
       <c r="I183" s="24" t="s">
-        <v>599</v>
+        <v>593</v>
       </c>
       <c r="J183" s="41" t="s">
         <v>439</v>
@@ -16188,7 +16215,7 @@
         <v>62</v>
       </c>
       <c r="S183" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T183" s="41"/>
       <c r="U183" s="24" t="s">
@@ -16201,7 +16228,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="184" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A184" s="24">
         <v>469</v>
       </c>
@@ -16266,7 +16293,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="185" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A185" s="24">
         <v>470</v>
       </c>
@@ -16289,10 +16316,10 @@
         <v>46090.710856481484</v>
       </c>
       <c r="H185" s="24" t="s">
-        <v>600</v>
+        <v>594</v>
       </c>
       <c r="I185" s="24" t="s">
-        <v>601</v>
+        <v>595</v>
       </c>
       <c r="J185" s="41" t="s">
         <v>439</v>
@@ -16322,7 +16349,7 @@
         <v>62</v>
       </c>
       <c r="S185" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T185" s="41"/>
       <c r="U185" s="24" t="s">
@@ -16335,76 +16362,76 @@
         <v>43</v>
       </c>
     </row>
-    <row r="186" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A186" s="24">
+    <row r="186" spans="1:23" s="60" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A186" s="51">
         <v>471</v>
       </c>
-      <c r="B186" s="24" t="s">
+      <c r="B186" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="C186" s="44" t="s">
+      <c r="C186" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="D186" s="24" t="s">
+      <c r="D186" s="51" t="s">
         <v>407</v>
       </c>
-      <c r="E186" s="38" t="s">
+      <c r="E186" s="53" t="s">
         <v>408</v>
       </c>
-      <c r="F186" s="40">
+      <c r="F186" s="54">
         <v>46090</v>
       </c>
-      <c r="G186" s="40">
-        <v>46090.479803240742</v>
-      </c>
-      <c r="H186" s="40" t="s">
-        <v>602</v>
-      </c>
-      <c r="I186" s="50" t="s">
-        <v>603</v>
-      </c>
-      <c r="J186" s="41" t="s">
+      <c r="G186" s="54">
+        <v>46100</v>
+      </c>
+      <c r="H186" s="54" t="s">
+        <v>594</v>
+      </c>
+      <c r="I186" s="55" t="s">
+        <v>595</v>
+      </c>
+      <c r="J186" s="56" t="s">
         <v>439</v>
       </c>
-      <c r="K186" s="41" t="s">
-        <v>440</v>
-      </c>
-      <c r="L186" s="41" t="s">
-        <v>440</v>
-      </c>
-      <c r="M186" s="41" t="s">
-        <v>224</v>
-      </c>
-      <c r="N186" s="41" t="s">
-        <v>224</v>
-      </c>
-      <c r="O186" s="41" t="s">
-        <v>440</v>
-      </c>
-      <c r="P186" s="41" t="s">
+      <c r="K186" s="56" t="s">
+        <v>440</v>
+      </c>
+      <c r="L186" s="56" t="s">
+        <v>440</v>
+      </c>
+      <c r="M186" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="N186" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="O186" s="56" t="s">
+        <v>440</v>
+      </c>
+      <c r="P186" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="Q186" s="41" t="s">
-        <v>224</v>
-      </c>
-      <c r="R186" s="41" t="s">
+      <c r="Q186" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="R186" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="S186" s="46" t="s">
-        <v>613</v>
-      </c>
-      <c r="T186" s="41"/>
-      <c r="U186" s="42" t="s">
-        <v>440</v>
-      </c>
-      <c r="V186" s="43" t="s">
-        <v>440</v>
-      </c>
-      <c r="W186" s="41" t="s">
+      <c r="S186" s="57" t="s">
+        <v>605</v>
+      </c>
+      <c r="T186" s="56"/>
+      <c r="U186" s="58" t="s">
+        <v>440</v>
+      </c>
+      <c r="V186" s="59" t="s">
+        <v>440</v>
+      </c>
+      <c r="W186" s="56" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="187" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A187" s="24">
         <v>472</v>
       </c>
@@ -16427,10 +16454,10 @@
         <v>46090.479803240742</v>
       </c>
       <c r="H187" s="40" t="s">
-        <v>604</v>
+        <v>596</v>
       </c>
       <c r="I187" s="50" t="s">
-        <v>605</v>
+        <v>597</v>
       </c>
       <c r="J187" s="41" t="s">
         <v>439</v>
@@ -16460,7 +16487,7 @@
         <v>62</v>
       </c>
       <c r="S187" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T187" s="41"/>
       <c r="U187" s="42" t="s">
@@ -16473,7 +16500,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="188" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A188" s="24">
         <v>473</v>
       </c>
@@ -16496,10 +16523,10 @@
         <v>46090.439305555556</v>
       </c>
       <c r="H188" s="40" t="s">
-        <v>606</v>
+        <v>598</v>
       </c>
       <c r="I188" s="50" t="s">
-        <v>607</v>
+        <v>599</v>
       </c>
       <c r="J188" s="41" t="s">
         <v>439</v>
@@ -16529,7 +16556,7 @@
         <v>62</v>
       </c>
       <c r="S188" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T188" s="41"/>
       <c r="U188" s="42" t="s">
@@ -16542,7 +16569,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="189" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A189" s="24">
         <v>474</v>
       </c>
@@ -16565,10 +16592,10 @@
         <v>46090.479814814818</v>
       </c>
       <c r="H189" s="40" t="s">
-        <v>608</v>
+        <v>600</v>
       </c>
       <c r="I189" s="50" t="s">
-        <v>609</v>
+        <v>601</v>
       </c>
       <c r="J189" s="41" t="s">
         <v>439</v>
@@ -16598,7 +16625,7 @@
         <v>62</v>
       </c>
       <c r="S189" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T189" s="41"/>
       <c r="U189" s="42" t="s">
@@ -16611,7 +16638,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="190" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A190" s="24">
         <v>475</v>
       </c>
@@ -16634,10 +16661,10 @@
         <v>46090.410671296297</v>
       </c>
       <c r="H190" s="40" t="s">
-        <v>610</v>
+        <v>602</v>
       </c>
       <c r="I190" s="50" t="s">
-        <v>611</v>
+        <v>603</v>
       </c>
       <c r="J190" s="41" t="s">
         <v>439</v>
@@ -16667,7 +16694,7 @@
         <v>62</v>
       </c>
       <c r="S190" s="46" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
       <c r="T190" s="41"/>
       <c r="U190" s="42" t="s">
@@ -16680,7 +16707,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="191" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A191" s="24">
         <v>476</v>
       </c>
@@ -16745,7 +16772,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="192" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A192" s="24">
         <v>477</v>
       </c>
@@ -16810,7 +16837,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="193" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A193" s="24">
         <v>478</v>
       </c>
@@ -20827,17 +20854,7 @@
       <c r="W745" s="27"/>
     </row>
   </sheetData>
-  <autoFilter ref="A9:W193" xr:uid="{00000000-0001-0000-0200-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="191"/>
-        <filter val="376"/>
-        <filter val="425"/>
-        <filter val="47"/>
-        <filter val="48"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A9:W193" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <mergeCells count="7">
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A2:B2"/>

</xml_diff>

<commit_message>
Fix test 470, 471
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#GASNETGROUPXX/gasnet/SaniPocket/V1.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#GASNETGROUPXX/gasnet/SaniPocket/V1.0/report-checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\simone.bettini\Desktop\temp\20260310_labelling_nazionale_LAB_LDO_RAD_RAP_RSA\SUBMISSION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8099B23F-36A3-4AB8-9D48-FAF2CDD9047B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9A9D681-2456-481A-BE24-E1352635E33B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3597" uniqueCount="616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3599" uniqueCount="620">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -2097,12 +2097,6 @@
     <t>2.16.840.1.113883.2.9.2.120.4.4.2149fb78666c205ac20b9bd2d882af037f0819429c691196eaa8054488c56c20.b1e50a4f99^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
-    <t>186d4bd4317b34bd4eb17bb71d8c93f8</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.50.4.5.30345.a54593994ef7b05118b20f6f168055ed4323b46afcc93e057bbd7d4b67748990.ee5036df1f^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>a49f4a815b0b475d41b46e79cd4427e1</t>
   </si>
   <si>
@@ -2161,6 +2155,24 @@
   </si>
   <si>
     <t>2.16.840.1.113883.2.9.2.50.4.5.50234.e5f4f4b379b1c6788d3ec0943e8129437c68075e18abd050c7932c56841ee5da.e5c5efa562^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>636968284009d6a651a2da3568329178</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.50.4.4.8da4985e6629cb97bac76de6d99aa1dfe928bc7deb2cc373a72e5d2c7e716a47.f9051590b8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-20T17:15:59Z</t>
+  </si>
+  <si>
+    <t>379ab31f45376d1fdacc4919f32b0324</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.50.4.5.30345.a54593994ef7b05118b20f6f168055ed4323b46afcc93e057bbd7d4b67748990.9221bfd030^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-03-20T17:38:00Z</t>
   </si>
 </sst>
 </file>
@@ -2170,7 +2182,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2299,6 +2311,13 @@
     <font>
       <b/>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -2675,7 +2694,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2869,6 +2888,37 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4356,7 +4406,7 @@
       </c>
       <c r="B2" s="63"/>
       <c r="C2" s="64" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="D2" s="65"/>
       <c r="F2" s="26"/>
@@ -4384,7 +4434,7 @@
       </c>
       <c r="B3" s="67"/>
       <c r="C3" s="64" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="D3" s="65"/>
       <c r="F3" s="26"/>
@@ -4410,7 +4460,7 @@
       <c r="A4" s="68"/>
       <c r="B4" s="69"/>
       <c r="C4" s="64" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="D4" s="65"/>
       <c r="F4" s="26"/>
@@ -4436,7 +4486,7 @@
       <c r="A5" s="70"/>
       <c r="B5" s="71"/>
       <c r="C5" s="64" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="D5" s="65"/>
       <c r="F5" s="26"/>
@@ -4711,7 +4761,7 @@
         <v>62</v>
       </c>
       <c r="S11" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T11" s="41"/>
       <c r="U11" s="42" t="s">
@@ -4780,7 +4830,7 @@
         <v>62</v>
       </c>
       <c r="S12" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T12" s="41"/>
       <c r="U12" s="42" t="s">
@@ -4914,7 +4964,7 @@
         <v>62</v>
       </c>
       <c r="S14" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T14" s="41"/>
       <c r="U14" s="42" t="s">
@@ -4983,7 +5033,7 @@
         <v>62</v>
       </c>
       <c r="S15" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T15" s="41"/>
       <c r="U15" s="42" t="s">
@@ -5247,7 +5297,7 @@
         <v>62</v>
       </c>
       <c r="S19" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T19" s="41"/>
       <c r="U19" s="42" t="s">
@@ -5316,7 +5366,7 @@
         <v>62</v>
       </c>
       <c r="S20" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T20" s="41"/>
       <c r="U20" s="42" t="s">
@@ -5450,7 +5500,7 @@
         <v>62</v>
       </c>
       <c r="S22" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T22" s="41"/>
       <c r="U22" s="42" t="s">
@@ -5519,7 +5569,7 @@
         <v>62</v>
       </c>
       <c r="S23" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T23" s="41"/>
       <c r="U23" s="42" t="s">
@@ -5779,7 +5829,7 @@
         <v>62</v>
       </c>
       <c r="S27" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T27" s="41"/>
       <c r="U27" s="42" t="s">
@@ -5844,7 +5894,7 @@
         <v>62</v>
       </c>
       <c r="S28" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T28" s="41"/>
       <c r="U28" s="42" t="s">
@@ -5974,7 +6024,7 @@
         <v>62</v>
       </c>
       <c r="S30" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T30" s="41"/>
       <c r="U30" s="42" t="s">
@@ -6039,7 +6089,7 @@
         <v>62</v>
       </c>
       <c r="S31" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T31" s="41"/>
       <c r="U31" s="42" t="s">
@@ -6303,7 +6353,7 @@
         <v>62</v>
       </c>
       <c r="S35" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T35" s="41"/>
       <c r="U35" s="42" t="s">
@@ -6372,7 +6422,7 @@
         <v>62</v>
       </c>
       <c r="S36" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T36" s="41"/>
       <c r="U36" s="42" t="s">
@@ -6441,7 +6491,7 @@
         <v>62</v>
       </c>
       <c r="S37" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T37" s="41"/>
       <c r="U37" s="42" t="s">
@@ -6510,7 +6560,7 @@
         <v>62</v>
       </c>
       <c r="S38" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T38" s="41"/>
       <c r="U38" s="42" t="s">
@@ -6579,7 +6629,7 @@
         <v>62</v>
       </c>
       <c r="S39" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T39" s="41"/>
       <c r="U39" s="42" t="s">
@@ -6648,7 +6698,7 @@
         <v>62</v>
       </c>
       <c r="S40" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T40" s="41"/>
       <c r="U40" s="42" t="s">
@@ -6717,7 +6767,7 @@
         <v>62</v>
       </c>
       <c r="S41" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T41" s="41"/>
       <c r="U41" s="42" t="s">
@@ -6786,7 +6836,7 @@
         <v>62</v>
       </c>
       <c r="S42" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T42" s="41"/>
       <c r="U42" s="42" t="s">
@@ -6855,7 +6905,7 @@
         <v>62</v>
       </c>
       <c r="S43" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T43" s="41"/>
       <c r="U43" s="42" t="s">
@@ -6924,7 +6974,7 @@
         <v>62</v>
       </c>
       <c r="S44" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T44" s="41"/>
       <c r="U44" s="42" t="s">
@@ -6993,7 +7043,7 @@
         <v>62</v>
       </c>
       <c r="S45" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T45" s="41"/>
       <c r="U45" s="42" t="s">
@@ -7062,7 +7112,7 @@
         <v>62</v>
       </c>
       <c r="S46" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T46" s="41"/>
       <c r="U46" s="42" t="s">
@@ -7131,7 +7181,7 @@
         <v>62</v>
       </c>
       <c r="S47" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T47" s="41"/>
       <c r="U47" s="42" t="s">
@@ -7200,7 +7250,7 @@
         <v>62</v>
       </c>
       <c r="S48" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T48" s="41"/>
       <c r="U48" s="42" t="s">
@@ -7269,7 +7319,7 @@
         <v>62</v>
       </c>
       <c r="S49" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T49" s="41"/>
       <c r="U49" s="42" t="s">
@@ -7338,7 +7388,7 @@
         <v>62</v>
       </c>
       <c r="S50" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T50" s="41"/>
       <c r="U50" s="42" t="s">
@@ -7407,7 +7457,7 @@
         <v>62</v>
       </c>
       <c r="S51" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T51" s="41"/>
       <c r="U51" s="42" t="s">
@@ -7476,7 +7526,7 @@
         <v>62</v>
       </c>
       <c r="S52" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T52" s="41"/>
       <c r="U52" s="42" t="s">
@@ -7545,7 +7595,7 @@
         <v>62</v>
       </c>
       <c r="S53" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T53" s="41"/>
       <c r="U53" s="42" t="s">
@@ -7614,7 +7664,7 @@
         <v>62</v>
       </c>
       <c r="S54" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T54" s="41"/>
       <c r="U54" s="42" t="s">
@@ -7683,7 +7733,7 @@
         <v>62</v>
       </c>
       <c r="S55" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T55" s="41"/>
       <c r="U55" s="42" t="s">
@@ -7752,7 +7802,7 @@
         <v>62</v>
       </c>
       <c r="S56" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T56" s="41"/>
       <c r="U56" s="42" t="s">
@@ -7821,7 +7871,7 @@
         <v>62</v>
       </c>
       <c r="S57" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T57" s="41"/>
       <c r="U57" s="42" t="s">
@@ -7890,7 +7940,7 @@
         <v>62</v>
       </c>
       <c r="S58" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T58" s="41"/>
       <c r="U58" s="42" t="s">
@@ -7959,7 +8009,7 @@
         <v>62</v>
       </c>
       <c r="S59" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T59" s="41"/>
       <c r="U59" s="42" t="s">
@@ -8028,7 +8078,7 @@
         <v>62</v>
       </c>
       <c r="S60" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T60" s="41"/>
       <c r="U60" s="42" t="s">
@@ -8097,7 +8147,7 @@
         <v>62</v>
       </c>
       <c r="S61" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T61" s="41"/>
       <c r="U61" s="42" t="s">
@@ -8166,7 +8216,7 @@
         <v>62</v>
       </c>
       <c r="S62" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T62" s="41"/>
       <c r="U62" s="42" t="s">
@@ -8235,7 +8285,7 @@
         <v>62</v>
       </c>
       <c r="S63" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T63" s="41"/>
       <c r="U63" s="42" t="s">
@@ -8304,7 +8354,7 @@
         <v>62</v>
       </c>
       <c r="S64" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T64" s="41"/>
       <c r="U64" s="42" t="s">
@@ -8373,7 +8423,7 @@
         <v>62</v>
       </c>
       <c r="S65" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T65" s="41"/>
       <c r="U65" s="42" t="s">
@@ -8442,7 +8492,7 @@
         <v>62</v>
       </c>
       <c r="S66" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T66" s="41"/>
       <c r="U66" s="42" t="s">
@@ -8511,7 +8561,7 @@
         <v>62</v>
       </c>
       <c r="S67" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T67" s="41"/>
       <c r="U67" s="42" t="s">
@@ -8580,7 +8630,7 @@
         <v>62</v>
       </c>
       <c r="S68" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T68" s="41"/>
       <c r="U68" s="42" t="s">
@@ -11704,7 +11754,7 @@
         <v>62</v>
       </c>
       <c r="S116" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T116" s="41"/>
       <c r="U116" s="42" t="s">
@@ -11773,7 +11823,7 @@
         <v>62</v>
       </c>
       <c r="S117" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T117" s="41"/>
       <c r="U117" s="42" t="s">
@@ -11842,7 +11892,7 @@
         <v>62</v>
       </c>
       <c r="S118" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T118" s="41"/>
       <c r="U118" s="42" t="s">
@@ -11911,7 +11961,7 @@
         <v>62</v>
       </c>
       <c r="S119" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T119" s="41"/>
       <c r="U119" s="42" t="s">
@@ -11980,7 +12030,7 @@
         <v>62</v>
       </c>
       <c r="S120" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T120" s="41"/>
       <c r="U120" s="42" t="s">
@@ -12049,7 +12099,7 @@
         <v>62</v>
       </c>
       <c r="S121" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T121" s="41"/>
       <c r="U121" s="42" t="s">
@@ -12118,7 +12168,7 @@
         <v>62</v>
       </c>
       <c r="S122" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T122" s="41"/>
       <c r="U122" s="42" t="s">
@@ -12187,7 +12237,7 @@
         <v>62</v>
       </c>
       <c r="S123" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T123" s="41"/>
       <c r="U123" s="42" t="s">
@@ -12256,7 +12306,7 @@
         <v>62</v>
       </c>
       <c r="S124" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T124" s="41"/>
       <c r="U124" s="42" t="s">
@@ -12325,7 +12375,7 @@
         <v>62</v>
       </c>
       <c r="S125" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T125" s="41"/>
       <c r="U125" s="42" t="s">
@@ -12394,7 +12444,7 @@
         <v>62</v>
       </c>
       <c r="S126" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T126" s="41"/>
       <c r="U126" s="42" t="s">
@@ -12463,7 +12513,7 @@
         <v>62</v>
       </c>
       <c r="S127" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T127" s="41"/>
       <c r="U127" s="42" t="s">
@@ -12532,7 +12582,7 @@
         <v>62</v>
       </c>
       <c r="S128" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T128" s="41"/>
       <c r="U128" s="42" t="s">
@@ -12601,7 +12651,7 @@
         <v>62</v>
       </c>
       <c r="S129" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T129" s="41"/>
       <c r="U129" s="42" t="s">
@@ -12670,7 +12720,7 @@
         <v>62</v>
       </c>
       <c r="S130" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T130" s="41"/>
       <c r="U130" s="42" t="s">
@@ -13683,7 +13733,7 @@
         <v>440</v>
       </c>
       <c r="J146" s="41" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="K146" s="41" t="s">
         <v>227</v>
@@ -13746,7 +13796,7 @@
         <v>440</v>
       </c>
       <c r="J147" s="41" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="K147" s="41" t="s">
         <v>227</v>
@@ -13840,7 +13890,7 @@
         <v>62</v>
       </c>
       <c r="S148" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T148" s="41"/>
       <c r="U148" s="42" t="s">
@@ -13909,7 +13959,7 @@
         <v>62</v>
       </c>
       <c r="S149" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T149" s="41"/>
       <c r="U149" s="42" t="s">
@@ -13922,72 +13972,72 @@
         <v>36</v>
       </c>
     </row>
-    <row r="150" spans="1:23" s="60" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A150" s="51">
+    <row r="150" spans="1:23" s="81" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A150" s="72">
         <v>419</v>
       </c>
-      <c r="B150" s="51" t="s">
+      <c r="B150" s="72" t="s">
         <v>34</v>
       </c>
-      <c r="C150" s="52" t="s">
+      <c r="C150" s="73" t="s">
         <v>239</v>
       </c>
-      <c r="D150" s="51" t="s">
+      <c r="D150" s="72" t="s">
         <v>242</v>
       </c>
-      <c r="E150" s="53" t="s">
+      <c r="E150" s="74" t="s">
         <v>267</v>
       </c>
-      <c r="F150" s="54">
+      <c r="F150" s="75">
         <v>46090</v>
       </c>
-      <c r="G150" s="54">
+      <c r="G150" s="75">
         <v>46100.38175925926</v>
       </c>
-      <c r="H150" s="54" t="s">
-        <v>614</v>
-      </c>
-      <c r="I150" s="55" t="s">
-        <v>615</v>
-      </c>
-      <c r="J150" s="56" t="s">
+      <c r="H150" s="75" t="s">
+        <v>612</v>
+      </c>
+      <c r="I150" s="76" t="s">
+        <v>613</v>
+      </c>
+      <c r="J150" s="77" t="s">
         <v>439</v>
       </c>
-      <c r="K150" s="56" t="s">
-        <v>440</v>
-      </c>
-      <c r="L150" s="56" t="s">
-        <v>440</v>
-      </c>
-      <c r="M150" s="56" t="s">
-        <v>224</v>
-      </c>
-      <c r="N150" s="56" t="s">
-        <v>224</v>
-      </c>
-      <c r="O150" s="56" t="s">
-        <v>440</v>
-      </c>
-      <c r="P150" s="56" t="s">
+      <c r="K150" s="77" t="s">
+        <v>440</v>
+      </c>
+      <c r="L150" s="77" t="s">
+        <v>440</v>
+      </c>
+      <c r="M150" s="77" t="s">
+        <v>224</v>
+      </c>
+      <c r="N150" s="77" t="s">
+        <v>224</v>
+      </c>
+      <c r="O150" s="77" t="s">
+        <v>440</v>
+      </c>
+      <c r="P150" s="77" t="s">
         <v>62</v>
       </c>
-      <c r="Q150" s="56" t="s">
-        <v>224</v>
-      </c>
-      <c r="R150" s="56" t="s">
+      <c r="Q150" s="77" t="s">
+        <v>224</v>
+      </c>
+      <c r="R150" s="77" t="s">
         <v>62</v>
       </c>
-      <c r="S150" s="57" t="s">
-        <v>605</v>
-      </c>
-      <c r="T150" s="56"/>
-      <c r="U150" s="58" t="s">
-        <v>440</v>
-      </c>
-      <c r="V150" s="59" t="s">
-        <v>440</v>
-      </c>
-      <c r="W150" s="56" t="s">
+      <c r="S150" s="78" t="s">
+        <v>603</v>
+      </c>
+      <c r="T150" s="77"/>
+      <c r="U150" s="79" t="s">
+        <v>440</v>
+      </c>
+      <c r="V150" s="80" t="s">
+        <v>440</v>
+      </c>
+      <c r="W150" s="77" t="s">
         <v>43</v>
       </c>
     </row>
@@ -14047,7 +14097,7 @@
         <v>62</v>
       </c>
       <c r="S151" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T151" s="41"/>
       <c r="U151" s="42" t="s">
@@ -14116,7 +14166,7 @@
         <v>62</v>
       </c>
       <c r="S152" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T152" s="41"/>
       <c r="U152" s="42" t="s">
@@ -14181,7 +14231,7 @@
         <v>62</v>
       </c>
       <c r="S153" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T153" s="41"/>
       <c r="U153" s="42" t="s">
@@ -14250,7 +14300,7 @@
         <v>62</v>
       </c>
       <c r="S154" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T154" s="41"/>
       <c r="U154" s="42" t="s">
@@ -14319,7 +14369,7 @@
         <v>62</v>
       </c>
       <c r="S155" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T155" s="41"/>
       <c r="U155" s="42" t="s">
@@ -14388,7 +14438,7 @@
         <v>62</v>
       </c>
       <c r="S156" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T156" s="41"/>
       <c r="U156" s="42" t="s">
@@ -14457,7 +14507,7 @@
         <v>62</v>
       </c>
       <c r="S157" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T157" s="41"/>
       <c r="U157" s="42" t="s">
@@ -14526,7 +14576,7 @@
         <v>62</v>
       </c>
       <c r="S158" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T158" s="41"/>
       <c r="U158" s="42" t="s">
@@ -14595,7 +14645,7 @@
         <v>62</v>
       </c>
       <c r="S159" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T159" s="41"/>
       <c r="U159" s="42" t="s">
@@ -14664,7 +14714,7 @@
         <v>62</v>
       </c>
       <c r="S160" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T160" s="41"/>
       <c r="U160" s="42" t="s">
@@ -14733,7 +14783,7 @@
         <v>62</v>
       </c>
       <c r="S161" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T161" s="41"/>
       <c r="U161" s="42" t="s">
@@ -14802,7 +14852,7 @@
         <v>62</v>
       </c>
       <c r="S162" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T162" s="41"/>
       <c r="U162" s="42" t="s">
@@ -14871,7 +14921,7 @@
         <v>62</v>
       </c>
       <c r="S163" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T163" s="41"/>
       <c r="U163" s="42" t="s">
@@ -14884,141 +14934,141 @@
         <v>43</v>
       </c>
     </row>
-    <row r="164" spans="1:23" s="60" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A164" s="51">
+    <row r="164" spans="1:23" s="81" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="72">
         <v>448</v>
       </c>
-      <c r="B164" s="51" t="s">
+      <c r="B164" s="72" t="s">
         <v>34</v>
       </c>
-      <c r="C164" s="52" t="s">
+      <c r="C164" s="73" t="s">
         <v>48</v>
       </c>
-      <c r="D164" s="51" t="s">
+      <c r="D164" s="72" t="s">
         <v>375</v>
       </c>
-      <c r="E164" s="53" t="s">
+      <c r="E164" s="74" t="s">
         <v>377</v>
       </c>
-      <c r="F164" s="54">
+      <c r="F164" s="75">
         <v>46090</v>
       </c>
-      <c r="G164" s="54">
+      <c r="G164" s="75">
         <v>46100</v>
       </c>
-      <c r="H164" s="54" t="s">
+      <c r="H164" s="75" t="s">
+        <v>608</v>
+      </c>
+      <c r="I164" s="76" t="s">
         <v>610</v>
       </c>
-      <c r="I164" s="55" t="s">
-        <v>612</v>
-      </c>
-      <c r="J164" s="56" t="s">
+      <c r="J164" s="77" t="s">
         <v>439</v>
       </c>
-      <c r="K164" s="56" t="s">
-        <v>440</v>
-      </c>
-      <c r="L164" s="56" t="s">
-        <v>440</v>
-      </c>
-      <c r="M164" s="56" t="s">
-        <v>224</v>
-      </c>
-      <c r="N164" s="56" t="s">
-        <v>224</v>
-      </c>
-      <c r="O164" s="56" t="s">
-        <v>440</v>
-      </c>
-      <c r="P164" s="56" t="s">
+      <c r="K164" s="77" t="s">
+        <v>440</v>
+      </c>
+      <c r="L164" s="77" t="s">
+        <v>440</v>
+      </c>
+      <c r="M164" s="77" t="s">
+        <v>224</v>
+      </c>
+      <c r="N164" s="77" t="s">
+        <v>224</v>
+      </c>
+      <c r="O164" s="77" t="s">
+        <v>440</v>
+      </c>
+      <c r="P164" s="77" t="s">
         <v>62</v>
       </c>
-      <c r="Q164" s="56" t="s">
-        <v>224</v>
-      </c>
-      <c r="R164" s="56" t="s">
+      <c r="Q164" s="77" t="s">
+        <v>224</v>
+      </c>
+      <c r="R164" s="77" t="s">
         <v>62</v>
       </c>
-      <c r="S164" s="57" t="s">
-        <v>605</v>
-      </c>
-      <c r="T164" s="56"/>
-      <c r="U164" s="58" t="s">
-        <v>440</v>
-      </c>
-      <c r="V164" s="59" t="s">
-        <v>440</v>
-      </c>
-      <c r="W164" s="56" t="s">
+      <c r="S164" s="78" t="s">
+        <v>603</v>
+      </c>
+      <c r="T164" s="77"/>
+      <c r="U164" s="79" t="s">
+        <v>440</v>
+      </c>
+      <c r="V164" s="80" t="s">
+        <v>440</v>
+      </c>
+      <c r="W164" s="77" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="165" spans="1:23" s="60" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A165" s="51">
+    <row r="165" spans="1:23" s="81" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A165" s="72">
         <v>449</v>
       </c>
-      <c r="B165" s="51" t="s">
+      <c r="B165" s="72" t="s">
         <v>34</v>
       </c>
-      <c r="C165" s="52" t="s">
+      <c r="C165" s="73" t="s">
         <v>48</v>
       </c>
-      <c r="D165" s="51" t="s">
+      <c r="D165" s="72" t="s">
         <v>376</v>
       </c>
-      <c r="E165" s="53" t="s">
+      <c r="E165" s="74" t="s">
         <v>378</v>
       </c>
-      <c r="F165" s="54">
+      <c r="F165" s="75">
         <v>46090</v>
       </c>
-      <c r="G165" s="54">
+      <c r="G165" s="75">
         <v>46100</v>
       </c>
-      <c r="H165" s="54" t="s">
-        <v>613</v>
-      </c>
-      <c r="I165" s="55" t="s">
+      <c r="H165" s="75" t="s">
         <v>611</v>
       </c>
-      <c r="J165" s="56" t="s">
+      <c r="I165" s="76" t="s">
+        <v>609</v>
+      </c>
+      <c r="J165" s="77" t="s">
         <v>439</v>
       </c>
-      <c r="K165" s="56" t="s">
-        <v>440</v>
-      </c>
-      <c r="L165" s="56" t="s">
-        <v>440</v>
-      </c>
-      <c r="M165" s="56" t="s">
-        <v>224</v>
-      </c>
-      <c r="N165" s="56" t="s">
-        <v>224</v>
-      </c>
-      <c r="O165" s="56" t="s">
-        <v>440</v>
-      </c>
-      <c r="P165" s="56" t="s">
+      <c r="K165" s="77" t="s">
+        <v>440</v>
+      </c>
+      <c r="L165" s="77" t="s">
+        <v>440</v>
+      </c>
+      <c r="M165" s="77" t="s">
+        <v>224</v>
+      </c>
+      <c r="N165" s="77" t="s">
+        <v>224</v>
+      </c>
+      <c r="O165" s="77" t="s">
+        <v>440</v>
+      </c>
+      <c r="P165" s="77" t="s">
         <v>62</v>
       </c>
-      <c r="Q165" s="56" t="s">
-        <v>224</v>
-      </c>
-      <c r="R165" s="56" t="s">
+      <c r="Q165" s="77" t="s">
+        <v>224</v>
+      </c>
+      <c r="R165" s="77" t="s">
         <v>62</v>
       </c>
-      <c r="S165" s="57" t="s">
-        <v>605</v>
-      </c>
-      <c r="T165" s="56"/>
-      <c r="U165" s="58" t="s">
-        <v>440</v>
-      </c>
-      <c r="V165" s="59" t="s">
-        <v>440</v>
-      </c>
-      <c r="W165" s="56" t="s">
+      <c r="S165" s="78" t="s">
+        <v>603</v>
+      </c>
+      <c r="T165" s="77"/>
+      <c r="U165" s="79" t="s">
+        <v>440</v>
+      </c>
+      <c r="V165" s="80" t="s">
+        <v>440</v>
+      </c>
+      <c r="W165" s="77" t="s">
         <v>36</v>
       </c>
     </row>
@@ -15078,7 +15128,7 @@
         <v>62</v>
       </c>
       <c r="S166" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T166" s="41"/>
       <c r="U166" s="42" t="s">
@@ -15147,7 +15197,7 @@
         <v>62</v>
       </c>
       <c r="S167" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T167" s="41"/>
       <c r="U167" s="42" t="s">
@@ -15216,7 +15266,7 @@
         <v>62</v>
       </c>
       <c r="S168" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T168" s="41"/>
       <c r="U168" s="42" t="s">
@@ -15675,7 +15725,7 @@
         <v>62</v>
       </c>
       <c r="S175" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T175" s="41"/>
       <c r="U175" s="42" t="s">
@@ -15744,7 +15794,7 @@
         <v>62</v>
       </c>
       <c r="S176" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T176" s="41"/>
       <c r="U176" s="24" t="s">
@@ -15813,7 +15863,7 @@
         <v>62</v>
       </c>
       <c r="S177" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T177" s="41"/>
       <c r="U177" s="24" t="s">
@@ -16077,7 +16127,7 @@
         <v>62</v>
       </c>
       <c r="S181" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T181" s="41"/>
       <c r="U181" s="24" t="s">
@@ -16146,7 +16196,7 @@
         <v>62</v>
       </c>
       <c r="S182" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T182" s="41"/>
       <c r="U182" s="24" t="s">
@@ -16179,7 +16229,7 @@
         <v>46090</v>
       </c>
       <c r="G183" s="24">
-        <v>46090.41065972222</v>
+        <v>46090.410659722198</v>
       </c>
       <c r="H183" s="24" t="s">
         <v>592</v>
@@ -16215,7 +16265,7 @@
         <v>62</v>
       </c>
       <c r="S183" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T183" s="41"/>
       <c r="U183" s="24" t="s">
@@ -16293,72 +16343,72 @@
         <v>43</v>
       </c>
     </row>
-    <row r="185" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A185" s="24">
+    <row r="185" spans="1:23" s="60" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A185" s="51">
         <v>470</v>
       </c>
-      <c r="B185" s="24" t="s">
+      <c r="B185" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="C185" s="44" t="s">
+      <c r="C185" s="52" t="s">
         <v>239</v>
       </c>
-      <c r="D185" s="24" t="s">
+      <c r="D185" s="51" t="s">
         <v>397</v>
       </c>
-      <c r="E185" s="38" t="s">
+      <c r="E185" s="53" t="s">
         <v>398</v>
       </c>
-      <c r="F185" s="24">
-        <v>46090</v>
-      </c>
-      <c r="G185" s="24">
-        <v>46090.710856481484</v>
-      </c>
-      <c r="H185" s="24" t="s">
-        <v>594</v>
-      </c>
-      <c r="I185" s="24" t="s">
-        <v>595</v>
-      </c>
-      <c r="J185" s="41" t="s">
+      <c r="F185" s="54">
+        <v>46101</v>
+      </c>
+      <c r="G185" s="54" t="s">
+        <v>619</v>
+      </c>
+      <c r="H185" s="51" t="s">
+        <v>617</v>
+      </c>
+      <c r="I185" s="51" t="s">
+        <v>618</v>
+      </c>
+      <c r="J185" s="56" t="s">
         <v>439</v>
       </c>
-      <c r="K185" s="41" t="s">
-        <v>440</v>
-      </c>
-      <c r="L185" s="24" t="s">
-        <v>440</v>
-      </c>
-      <c r="M185" s="41" t="s">
-        <v>224</v>
-      </c>
-      <c r="N185" s="41" t="s">
-        <v>224</v>
-      </c>
-      <c r="O185" s="41" t="s">
-        <v>440</v>
-      </c>
-      <c r="P185" s="41" t="s">
+      <c r="K185" s="56" t="s">
+        <v>440</v>
+      </c>
+      <c r="L185" s="51" t="s">
+        <v>440</v>
+      </c>
+      <c r="M185" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="N185" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="O185" s="56" t="s">
+        <v>440</v>
+      </c>
+      <c r="P185" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="Q185" s="41" t="s">
-        <v>224</v>
-      </c>
-      <c r="R185" s="41" t="s">
+      <c r="Q185" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="R185" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="S185" s="46" t="s">
-        <v>605</v>
-      </c>
-      <c r="T185" s="41"/>
-      <c r="U185" s="24" t="s">
-        <v>440</v>
-      </c>
-      <c r="V185" s="24" t="s">
-        <v>440</v>
-      </c>
-      <c r="W185" s="24" t="s">
+      <c r="S185" s="57" t="s">
+        <v>603</v>
+      </c>
+      <c r="T185" s="56"/>
+      <c r="U185" s="51" t="s">
+        <v>440</v>
+      </c>
+      <c r="V185" s="51" t="s">
+        <v>440</v>
+      </c>
+      <c r="W185" s="51" t="s">
         <v>43</v>
       </c>
     </row>
@@ -16379,16 +16429,16 @@
         <v>408</v>
       </c>
       <c r="F186" s="54">
-        <v>46090</v>
-      </c>
-      <c r="G186" s="54">
-        <v>46100</v>
+        <v>46101</v>
+      </c>
+      <c r="G186" s="54" t="s">
+        <v>616</v>
       </c>
       <c r="H186" s="54" t="s">
-        <v>594</v>
+        <v>614</v>
       </c>
       <c r="I186" s="55" t="s">
-        <v>595</v>
+        <v>615</v>
       </c>
       <c r="J186" s="56" t="s">
         <v>439</v>
@@ -16418,7 +16468,7 @@
         <v>62</v>
       </c>
       <c r="S186" s="57" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T186" s="56"/>
       <c r="U186" s="58" t="s">
@@ -16454,10 +16504,10 @@
         <v>46090.479803240742</v>
       </c>
       <c r="H187" s="40" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="I187" s="50" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="J187" s="41" t="s">
         <v>439</v>
@@ -16487,7 +16537,7 @@
         <v>62</v>
       </c>
       <c r="S187" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T187" s="41"/>
       <c r="U187" s="42" t="s">
@@ -16523,10 +16573,10 @@
         <v>46090.439305555556</v>
       </c>
       <c r="H188" s="40" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="I188" s="50" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="J188" s="41" t="s">
         <v>439</v>
@@ -16556,7 +16606,7 @@
         <v>62</v>
       </c>
       <c r="S188" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T188" s="41"/>
       <c r="U188" s="42" t="s">
@@ -16592,10 +16642,10 @@
         <v>46090.479814814818</v>
       </c>
       <c r="H189" s="40" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="I189" s="50" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="J189" s="41" t="s">
         <v>439</v>
@@ -16625,7 +16675,7 @@
         <v>62</v>
       </c>
       <c r="S189" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T189" s="41"/>
       <c r="U189" s="42" t="s">
@@ -16661,10 +16711,10 @@
         <v>46090.410671296297</v>
       </c>
       <c r="H190" s="40" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="I190" s="50" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="J190" s="41" t="s">
         <v>439</v>
@@ -16694,7 +16744,7 @@
         <v>62</v>
       </c>
       <c r="S190" s="46" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T190" s="41"/>
       <c r="U190" s="42" t="s">
@@ -16966,7 +17016,7 @@
       <c r="F197" s="26"/>
       <c r="G197" s="26"/>
       <c r="H197" s="26"/>
-      <c r="I197" s="26"/>
+      <c r="I197" s="82"/>
       <c r="J197" s="27"/>
       <c r="K197" s="27"/>
       <c r="L197" s="27"/>
@@ -23124,6 +23174,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BE9A258ADBC3EC4CBEB1E2AB9909207A" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0284f501378927579289f00316ec8a74">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="295b7897-c886-40bf-9750-5782b814c3e4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b47213d65be806e283915cff374a7eef" ns2:_="">
     <xsd:import namespace="295b7897-c886-40bf-9750-5782b814c3e4"/>
@@ -23267,12 +23323,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -23283,6 +23333,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7568E770-0BC4-46AF-B6C6-958AE21C8F7F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -23300,23 +23367,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>

</xml_diff>